<commit_message>
CharacterTable 이미지 URL 최신화 (v0.6.2)
인격 이미지(일반/각성/프로필)와 스킬1/2/3 아이콘 URL을 최신 데이터로 갱신.
기존에 64개 인격에서 스킬 아이콘 3개가 동일하게 나오던 문제도 이번 업데이트로 해결됨.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CharacterTable.xlsx
+++ b/CharacterTable.xlsx
@@ -506,7 +506,11 @@
           <t>참격</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/The%20House%20of%20Spiders%20The%20Thumb%20Apprentice/1071601_1.png</t>
+        </is>
+      </c>
       <c r="O2" t="inlineStr">
         <is>
           <t>콜피 소타니</t>
@@ -522,7 +526,11 @@
           <t>참격</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/The%20House%20of%20Spiders%20The%20Thumb%20Apprentice/1071602_2.png</t>
+        </is>
+      </c>
       <c r="S2" t="inlineStr">
         <is>
           <t>카치아토레</t>
@@ -540,7 +548,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/The%20House%20of%20Spiders%20The%20Thumb%20Apprentice/1071603%202.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/The%20House%20of%20Spiders%20The%20Thumb%20Apprentice/1071603.png</t>
         </is>
       </c>
       <c r="W2" t="n">
@@ -625,11 +633,7 @@
           <t>참격</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/The%20House%20of%20Spiders%20The%20Thumb%20Nursefather/1091604.png</t>
-        </is>
-      </c>
+      <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr">
         <is>
           <t>기꺼이 이 탄환으로 꿰뚫어주지</t>
@@ -645,11 +649,7 @@
           <t>참격</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/The%20House%20of%20Spiders%20The%20Thumb%20Nursefather/1091601.png</t>
-        </is>
-      </c>
+      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
           <t>세치오나투라 디 엘레판테</t>
@@ -665,11 +665,7 @@
           <t>참격</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/The%20House%20of%20Spiders%20The%20Thumb%20Nursefather/1091603.png</t>
-        </is>
-      </c>
+      <c r="V3" t="inlineStr"/>
       <c r="W3" t="n">
         <v>4</v>
       </c>
@@ -750,7 +746,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/S%20Corp.%20Ch'unokkun/1061501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Constricting_Ohra_Bonds_Hong_Lu_Icon.png/74px-Constricting_Ohra_Bonds_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -770,7 +766,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/S%20Corp.%20Ch'unokkun/1061501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Avulsion_Slash_Hong_Lu_Icon.png/74px-Avulsion_Slash_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -790,7 +786,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/S%20Corp.%20Ch'unokkun/1061501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Hunter%27s_Scouring_Hong_Lu_Icon.png/74px-Hunter%27s_Scouring_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="W4" t="n">
@@ -873,7 +869,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/LCD%20OSIR%20Team/1081501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Rending_Arts_Ishmael_Icon.png/74px-Rending_Arts_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -893,7 +889,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/LCD%20OSIR%20Team/1081501_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Acupuncture_Ishmael_Icon.png/74px-Acupuncture_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -913,7 +909,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/LCD%20OSIR%20Team/1081501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Lucent_Rippling_Flame_Ishmael_Icon.png/74px-Lucent_Rippling_Flame_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="W5" t="n">
@@ -1020,7 +1016,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/The%20House%20of%20Spiders%20The%20Middle%20Nursefather/1111501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Outis/The%20House%20of%20Spiders%20The%20Middle%20Nursefather/1111502.png</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1040,7 +1036,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/The%20House%20of%20Spiders%20The%20Middle%20Nursefather/1111501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Outis/The%20House%20of%20Spiders%20The%20Middle%20Nursefather/1111503.png</t>
         </is>
       </c>
       <c r="W6" t="n">
@@ -1127,7 +1123,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Blade%20of%20the%20House%20of%20Spiders/1041501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Tripleslash_%E4%B8%89%E9%80%A3_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Tripleslash_%E4%B8%89%E9%80%A3_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -1147,7 +1143,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Blade%20of%20the%20House%20of%20Spiders/1041501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Tripleslash_-_Echoshear_%E4%B8%89%E9%80%A3_-_%E6%AE%98_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Tripleslash_-_Echoshear_%E4%B8%89%E9%80%A3_-_%E6%AE%98_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1167,7 +1163,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Blade%20of%20the%20House%20of%20Spiders/1041501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Rend_Space_%E7%A9%BA%E9%96%93%E6%96%AC_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Rend_Space_%E7%A9%BA%E9%96%93%E6%96%AC_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="W7" t="n">
@@ -1250,7 +1246,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/The%20Middle%20Big%20Brother/1071501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Kicking_Heathcliff_Icon.png/74px-Kicking_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -1270,7 +1266,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/The%20Middle%20Big%20Brother/1071501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Watch_Your_Back%21_Heathcliff_Icon.png/74px-Watch_Your_Back%21_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1290,7 +1286,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/The%20Middle%20Big%20Brother/1071501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/MY_HAIR_COUPOOOOOOOOOOONS%21%21%21%21_Heathcliff_Icon.png/74px-MY_HAIR_COUPOOOOOOOOOOONS%21%21%21%21_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="W8" t="n">
@@ -1373,7 +1369,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/The%20Ring%20Fauvist%20Student/1051501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Rough_Portrayal_Meursault_Icon.png/74px-Rough_Portrayal_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1393,7 +1389,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/The%20Ring%20Fauvist%20Student/1051501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Visceral_Strokes_Meursault_Icon.png/74px-Visceral_Strokes_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1413,7 +1409,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/The%20Ring%20Fauvist%20Student/1051501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Le_Fauvisme_-_Reveal_Submission_Meursault_Icon.png/74px-Le_Fauvisme_-_Reveal_Submission_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="W9" t="n">
@@ -1496,7 +1492,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/The%20Ring%20Fauvist%20Docent/1091501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Vehement_Overpainting_Rodion_Icon.png/74px-Vehement_Overpainting_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1516,7 +1512,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/The%20Ring%20Fauvist%20Docent/1091501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Expression_of_Primary_Colors_Rodion_Icon.png/74px-Expression_of_Primary_Colors_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1536,7 +1532,7 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/The%20Ring%20Fauvist%20Docent/1091501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Le_Fauvisme_-_D%C3%A9cha%C3%AEnement_Brutal_Rodion_Icon.png/74px-Le_Fauvisme_-_D%C3%A9cha%C3%AEnement_Brutal_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="W10" t="n">
@@ -1643,7 +1639,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/The%20House%20of%20Spiders%20The%20Ring%20Apprentice/1021501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Faust/The%20House%20of%20Spiders%20The%20Ring%20Apprentice/1021502.png</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1663,7 +1659,7 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/The%20House%20of%20Spiders%20The%20Ring%20Apprentice/1021501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Faust/The%20House%20of%20Spiders%20The%20Ring%20Apprentice/1021503.png</t>
         </is>
       </c>
       <c r="W11" t="n">
@@ -1770,7 +1766,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/The%20House%20of%20Spiders%20The%20Ring%20Nursefather/1061401.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/The%20House%20of%20Spiders%20The%20Ring%20Nursefather/1061402.png</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1790,7 +1786,7 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/The%20House%20of%20Spiders%20The%20Ring%20Nursefather/1061401.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/The%20House%20of%20Spiders%20The%20Ring%20Nursefather/1061403.png</t>
         </is>
       </c>
       <c r="W12" t="n">
@@ -1873,7 +1869,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/LCE%20E.G.O%20AEDD/1121501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/LCE%20E.G.O%20AEDD/1121501_1.png</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1893,7 +1889,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/LCE%20E.G.O%20AEDD/1121501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/LCE%20E.G.O%20AEDD/1121502_2.png</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1913,7 +1909,7 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/LCE%20E.G.O%20AEDD/1121501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/LCE%20E.G.O%20AEDD/1121503.png</t>
         </is>
       </c>
       <c r="W13" t="n">
@@ -2016,7 +2012,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Lobotomy%20E.G.O%20Faint%20Aroma%20%26%20Solitude/1041401.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Lobotomy%20E.G.O%20Faint%20Aroma%20%26%20Solitude/1041402_2.png</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -2036,7 +2032,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Lobotomy%20E.G.O%20Faint%20Aroma%20%26%20Solitude/1041401.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Lobotomy%20E.G.O%20Faint%20Aroma%20%26%20Solitude/1041403.png</t>
         </is>
       </c>
       <c r="W14" t="n">
@@ -2119,7 +2115,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Lobotomy%20E.G.O%20Hornet%20%E3%80%90Alteration%E3%80%91/1051401.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Lobotomy%20E.G.O%20Hornet%20%E3%80%90Alteration%E3%80%91/1051401_1.png</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -2139,7 +2135,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Lobotomy%20E.G.O%20Hornet%20%E3%80%90Alteration%E3%80%91/1051401.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Lobotomy%20E.G.O%20Hornet%20%E3%80%90Alteration%E3%80%91/1051402_2.png</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2159,7 +2155,7 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Lobotomy%20E.G.O%20Hornet%20%E3%80%90Alteration%E3%80%91/1051401.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Lobotomy%20E.G.O%20Hornet%20%E3%80%90Alteration%E3%80%91/1051403_3.png</t>
         </is>
       </c>
       <c r="W15" t="n">
@@ -2246,7 +2242,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/The%20House%20of%20Spiders%20The%20Index%20Nursefather/1011501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/The%20House%20of%20Spiders%20The%20Index%20Nursefather/1011501_1.png</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -2266,7 +2262,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/The%20House%20of%20Spiders%20The%20Index%20Nursefather/1011501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/The%20House%20of%20Spiders%20The%20Index%20Nursefather/1011502_2.png</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2286,7 +2282,7 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/The%20House%20of%20Spiders%20The%20Index%20Nursefather/1011501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/The%20House%20of%20Spiders%20The%20Index%20Nursefather/1011503.png</t>
         </is>
       </c>
       <c r="W16" t="n">
@@ -2369,7 +2365,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/The%20House%20of%20Spiders%20The%20Pinky%20Apprentice/1101501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/The%20House%20of%20Spiders%20The%20Pinky%20Apprentice/1101501_1.png</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -2389,7 +2385,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/The%20House%20of%20Spiders%20The%20Pinky%20Apprentice/1101501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/The%20House%20of%20Spiders%20The%20Pinky%20Apprentice/1101502_2.png</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2409,7 +2405,7 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/The%20House%20of%20Spiders%20The%20Pinky%20Apprentice/1101501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/The%20House%20of%20Spiders%20The%20Pinky%20Apprentice/1101503_3.png</t>
         </is>
       </c>
       <c r="W17" t="n">
@@ -2492,7 +2488,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Lobotomy%20E.G.O%20Lamp/1121401.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Lobotomy%20E.G.O%20Lamp/1121401_1.png</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -2512,7 +2508,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Lobotomy%20E.G.O%20Lamp/1121401.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Lobotomy%20E.G.O%20Lamp/1121402_2.png</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2532,7 +2528,7 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Lobotomy%20E.G.O%20Lamp/1121401.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Lobotomy%20E.G.O%20Lamp/1121403_3.png</t>
         </is>
       </c>
       <c r="W18" t="n">
@@ -2619,7 +2615,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>https://cdn.discordapp.com/avatars/774965401707872257/a57c5805eb0e2ec936fcdf5f9fc8ef86.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/The%20House%20of%20Spiders%20The%20Middle%20Apprentice/1081401_1.png</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -2639,7 +2635,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>https://cdn.discordapp.com/avatars/774965401707872257/a57c5805eb0e2ec936fcdf5f9fc8ef86.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/The%20House%20of%20Spiders%20The%20Middle%20Apprentice/1081402_2.png</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2659,7 +2655,7 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>https://cdn.discordapp.com/avatars/774965401707872257/a57c5805eb0e2ec936fcdf5f9fc8ef86.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/The%20House%20of%20Spiders%20The%20Middle%20Apprentice/1081403_3.png</t>
         </is>
       </c>
       <c r="W19" t="n">
@@ -2762,7 +2758,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/The%20Index%20Proxy%20-%20Effloresced%20E.G.O%20Procuration/1031401.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/The%20Index%20Proxy%20-%20Effloresced%20E.G.O%20Procuration/1031402.png</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2782,7 +2778,7 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/The%20Index%20Proxy%20-%20Effloresced%20E.G.O%20Procuration/1031401.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/The%20Index%20Proxy%20-%20Effloresced%20E.G.O%20Procuration/1031403.png</t>
         </is>
       </c>
       <c r="W20" t="n">
@@ -2865,7 +2861,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/The%20Index%20Proselyte%20%E3%80%90Paper%20Slip%E3%80%91/1021401.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Faust/The%20Index%20Proselyte%20%E3%80%90Paper%20Slip%E3%80%91/1021401_1.png</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -2885,7 +2881,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/The%20Index%20Proselyte%20%E3%80%90Paper%20Slip%E3%80%91/1021401.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Faust/The%20Index%20Proselyte%20%E3%80%90Paper%20Slip%E3%80%91/1021402_2.png</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2905,7 +2901,7 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/The%20Index%20Proselyte%20%E3%80%90Paper%20Slip%E3%80%91/1021401.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Faust/The%20Index%20Proselyte%20%E3%80%90Paper%20Slip%E3%80%91/1021403_3.png</t>
         </is>
       </c>
       <c r="W21" t="n">
@@ -2988,7 +2984,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/LCA%20Udjat%20Vanguard%20Team%203%20Leader/1111401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Khopesh_Swordplay_Outis_Icon.png/74px-Khopesh_Swordplay_Outis_Icon.png</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -3008,7 +3004,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/LCA%20Udjat%20Vanguard%20Team%203%20Leader/1111401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Mirage_Incision_Outis_Icon.png/74px-Mirage_Incision_Outis_Icon.png</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -3028,7 +3024,7 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/LCA%20Udjat%20Vanguard%20Team%203%20Leader/1111401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/The_Vanguard_will_See_it_Down_Outis_Icon.png/74px-The_Vanguard_will_See_it_Down_Outis_Icon.png</t>
         </is>
       </c>
       <c r="W22" t="n">
@@ -3111,7 +3107,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/R%20Corp.%204th%20Pack%20Reindeer/1091401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Energy_Strike_-_%27That%27s_What_You_Get_For_Giving_Us_Holiday_Shifts%21%27_Rodion_Icon.png/74px-Energy_Strike_-_%27That%27s_What_You_Get_For_Giving_Us_Holiday_Shifts%21%27_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -3131,7 +3127,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/R%20Corp.%204th%20Pack%20Reindeer/1091401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Concentration_-_%27Burst_and_Pop_with_Christmas_Colors%21%27_Rodion_Icon.png/74px-Concentration_-_%27Burst_and_Pop_with_Christmas_Colors%21%27_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -3151,7 +3147,7 @@
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/R%20Corp.%204th%20Pack%20Reindeer/1091401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Mind_Whip_-_%27Ahaha..._Look%2C_Everyone%21_We%27re_the_Fireworks_this_Christmas%21%27_Rodion_Icon.png/74px-Mind_Whip_-_%27Ahaha..._Look%2C_Everyone%21_We%27re_the_Fireworks_this_Christmas%21%27_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="W23" t="n">
@@ -3234,7 +3230,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Drifting%20Blade%20of%20Hongyuan/1041301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Hey%2C_Back_Off_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Hey%2C_Back_Off_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -3254,7 +3250,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Drifting%20Blade%20of%20Hongyuan/1041301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Engraved_in_Flesh_and_Bone_%E9%8A%98%E8%82%8C%E9%8F%A4%E9%AA%A8_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Engraved_in_Flesh_and_Bone_%E9%8A%98%E8%82%8C%E9%8F%A4%E9%AA%A8_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3274,7 +3270,7 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Drifting%20Blade%20of%20Hongyuan/1041301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Aiding_Strike_%E5%8A%A0%E6%96%A5%E6%88%91%E6%8F%B4_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Aiding_Strike_%E5%8A%A0%E6%96%A5%E6%88%91%E6%8F%B4_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="W24" t="n">
@@ -3357,7 +3353,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/Heishou%20Pack%20-%20Wei%20Branch/1031301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Breakthrough_Don_Quixote_Icon.png/74px-Breakthrough_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -3377,7 +3373,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/Heishou%20Pack%20-%20Wei%20Branch/1031301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Seize_the_Momentum%2C_Shatter_the_Wall_Don_Quixote_Icon.png/74px-Seize_the_Momentum%2C_Shatter_the_Wall_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3397,7 +3393,7 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/Heishou%20Pack%20-%20Wei%20Branch/1031301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Crushing_Horns_%E7%A0%B4%E7%A2%8E%E8%A7%92_Don_Quixote_Icon.png/74px-Crushing_Horns_%E7%A0%B4%E7%A2%8E%E8%A7%92_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="W25" t="n">
@@ -3480,7 +3476,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Heishou%20Pack%20-%20You%20Branch%20Adept/1071401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Peck_%27em_Heathcliff_Icon.png/74px-Peck_%27em_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -3500,7 +3496,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Heishou%20Pack%20-%20You%20Branch%20Adept/1071401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Mutilating_Talons_Heathcliff_Icon.png/74px-Mutilating_Talons_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3520,7 +3516,7 @@
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Heishou%20Pack%20-%20You%20Branch%20Adept/1071401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Bloodflame_Massacre_%E8%A1%80%E7%82%8E%E4%BA%82%E8%88%9E_Heathcliff_Icon.png/74px-Bloodflame_Massacre_%E8%A1%80%E7%82%8E%E4%BA%82%E8%88%9E_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="W26" t="n">
@@ -3603,7 +3599,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Jeong_s%20Office%20Rep/1081301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Tsuru-giri_-%E9%B6%B4%E6%96%AC%E3%82%8A-_Ishmael_Icon.png/74px-Tsuru-giri_-%E9%B6%B4%E6%96%AC%E3%82%8A-_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
@@ -3623,7 +3619,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Jeong_s%20Office%20Rep/1081301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Susuki_Misdirection_Ishmael_Icon.png/74px-Susuki_Misdirection_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3643,7 +3639,7 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Jeong_s%20Office%20Rep/1081301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Sakura-sen_-%E6%A1%9C%E9%96%83-_Ishmael_Icon.png/74px-Sakura-sen_-%E6%A1%9C%E9%96%83-_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="W27" t="n">
@@ -3746,7 +3742,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Night%20Awls%20Capitano/1121301.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Night%20Awls%20Capitano/1121302_2.png</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3766,7 +3762,7 @@
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Night%20Awls%20Capitano/1121301.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Night%20Awls%20Capitano/1121303.png</t>
         </is>
       </c>
       <c r="W28" t="n">
@@ -3849,7 +3845,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/The%20Prince%20of%20La%20Manchaland/1051301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/March_Conductor_Meursault_Icon.png/74px-March_Conductor_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
@@ -3869,7 +3865,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/The%20Prince%20of%20La%20Manchaland/1051301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Responsibility_to_Rebuild_Meursault_Icon.png/74px-Responsibility_to_Rebuild_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3889,7 +3885,7 @@
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/The%20Prince%20of%20La%20Manchaland/1051301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Let_us_wear_the_coagulated_mantle_of_blood._Meursault_Icon.png/74px-Let_us_wear_the_coagulated_mantle_of_blood._Meursault_Icon.png</t>
         </is>
       </c>
       <c r="W29" t="n">
@@ -3972,7 +3968,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/W%20Corp.%20L4%20Cleanup%20Agent%20-%20CCA/1071301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Congestion_Cleanup_Heathcliff_Icon.png/74px-Congestion_Cleanup_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -3992,7 +3988,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/W%20Corp.%20L4%20Cleanup%20Agent%20-%20CCA/1071301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Boost_Elbow_Blade_Heathcliff_Icon.png/74px-Boost_Elbow_Blade_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -4012,7 +4008,7 @@
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/W%20Corp.%20L4%20Cleanup%20Agent%20-%20CCA/1071301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Rip_Space_-_CCA_Overdrive_Heathcliff_Icon.png/74px-Rip_Space_-_CCA_Overdrive_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="W30" t="n">
@@ -4095,7 +4091,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Shi%20Assoc.%20East%20Section%203/1021301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Cleave_Faust_Icon.png/74px-Cleave_Faust_Icon.png</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -4115,7 +4111,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Shi%20Assoc.%20East%20Section%203/1021301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Positioning_Maneuver_Faust_Icon.png/74px-Positioning_Maneuver_Faust_Icon.png</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -4135,7 +4131,7 @@
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Shi%20Assoc.%20East%20Section%203/1021301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Glimmering_Bow_%E5%BC%93%E9%96%83_Faust_Icon.png/74px-Glimmering_Bow_%E5%BC%93%E9%96%83_Faust_Icon.png</t>
         </is>
       </c>
       <c r="W31" t="n">
@@ -4238,7 +4234,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/N%20Corp.%20E.G.O%20Contempt%2C%20Awe/1041201.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/N%20Corp.%20E.G.O%20Contempt%2C%20Awe/1041202.png</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -4258,7 +4254,7 @@
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/N%20Corp.%20E.G.O%20Contempt%2C%20Awe/1041201.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/N%20Corp.%20E.G.O%20Contempt%2C%20Awe/1041203.png</t>
         </is>
       </c>
       <c r="W32" t="n">
@@ -4341,7 +4337,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>https://cdn.discordapp.com/avatars/1513117038938427532/db46a5402bbb67422eda3ac23817693d.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Cut_Down_and_Trample_Yi_Sang_Icon.png/74px-Cut_Down_and_Trample_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -4361,7 +4357,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Heishou%20Pack%20-%20Wu%20Branch/1011403%202.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Crescent_Blade_Strike_-%E6%9C%88%E5%88%80%E6%93%8A-_Yi_Sang_Icon.png/74px-Crescent_Blade_Strike_-%E6%9C%88%E5%88%80%E6%93%8A-_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -4381,7 +4377,7 @@
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Heishou%20Pack%20-%20Wu%20Branch/1011403%202.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Cavalry%27s_Vanguard_Charge_Yi_Sang_Icon.png/74px-Cavalry%27s_Vanguard_Charge_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="W33" t="n">
@@ -4464,7 +4460,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Heishou%20Pack%20-%20You%20Branch/1101401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Oh%2C_Let_the_Smell_of_Burning_Blood%E2%80%A6_Sinclair_Icon.png/74px-Oh%2C_Let_the_Smell_of_Burning_Blood%E2%80%A6_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
@@ -4484,7 +4480,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Heishou%20Pack%20-%20You%20Branch/1101401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/%E2%80%A6_Fuel_My_Rampage._Sinclair_Icon.png/74px-%E2%80%A6_Fuel_My_Rampage._Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4504,7 +4500,7 @@
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Heishou%20Pack%20-%20You%20Branch/1101401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Bloodflame_Massacre_-%E8%A1%80%E7%82%8E%E4%BA%82%E8%88%9E-_Sinclair_Icon.png/74px-Bloodflame_Massacre_-%E8%A1%80%E7%82%8E%E4%BA%82%E8%88%9E-_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="W34" t="n">
@@ -4587,7 +4583,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/The%20Lord%20of%20Hongyuan/1061301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/I_Wish_to_Open_the_Path_Hong_Lu_Icon.png/74px-I_Wish_to_Open_the_Path_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
@@ -4607,7 +4603,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/The%20Lord%20of%20Hongyuan/1061301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Tarnished_Blood%27s_Absolute_Cleaver_of_Ambitions_-%E6%B1%9A%E8%A1%80%E7%B5%95%E5%BF%97%E7%AB%9F%E6%88%90-_Hong_Lu_Icon.png/74px-Tarnished_Blood%27s_Absolute_Cleaver_of_Ambitions_-%E6%B1%9A%E8%A1%80%E7%B5%95%E5%BF%97%E7%AB%9F%E6%88%90-_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4627,7 +4623,7 @@
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/The%20Lord%20of%20Hongyuan/1061301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Answer_Me%2C_Heishou_Packs_Hong_Lu_Icon.png/74px-Answer_Me%2C_Heishou_Packs_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="W35" t="n">
@@ -4706,7 +4702,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/T%20Corp.%20Class%203%20VDCU%20Staff/1111301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Prepare_to_Collect_Outis_Icon.png/74px-Prepare_to_Collect_Outis_Icon.png</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
@@ -4726,7 +4722,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/T%20Corp.%20Class%203%20VDCU%20Staff/1111301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/T_Corp._Microcavity_Module_Outis_Icon.png/74px-T_Corp._Microcavity_Module_Outis_Icon.png</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4746,7 +4742,7 @@
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/T%20Corp.%20Class%203%20VDCU%20Staff/1111301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/T-3_Collector_Mace_Max_Activation_Outis_Icon.png/74px-T-3_Collector_Mace_Max_Activation_Outis_Icon.png</t>
         </is>
       </c>
       <c r="W36" t="n">
@@ -4849,7 +4845,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/Lobotomy%20E.G.O%20In%20the%20Name%20of%20Love%20and%20Hate/1031201.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/Lobotomy%20E.G.O%20In%20the%20Name%20of%20Love%20and%20Hate/1031202.png</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4869,7 +4865,7 @@
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/Lobotomy%20E.G.O%20In%20the%20Name%20of%20Love%20and%20Hate/1031201.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/Lobotomy%20E.G.O%20In%20the%20Name%20of%20Love%20and%20Hate/1031203.png</t>
         </is>
       </c>
       <c r="W37" t="n">
@@ -4972,7 +4968,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Lobotomy%20E.G.O%20The%20Sword%20Sharpened%20With%20Tears/1091301.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Lobotomy%20E.G.O%20The%20Sword%20Sharpened%20With%20Tears/1091302.png</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4992,7 +4988,7 @@
       </c>
       <c r="V38" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Lobotomy%20E.G.O%20The%20Sword%20Sharpened%20With%20Tears/1091301.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Lobotomy%20E.G.O%20The%20Sword%20Sharpened%20With%20Tears/1091303.png</t>
         </is>
       </c>
       <c r="W38" t="n">
@@ -5075,7 +5071,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/N%20Corp.%20E.G.O%20Fell%20Bullet/1011301.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/N%20Corp.%20E.G.O%20Fell%20Bullet/1011301_1.png</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
@@ -5095,7 +5091,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/N%20Corp.%20E.G.O%20Fell%20Bullet/1011301.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/N%20Corp.%20E.G.O%20Fell%20Bullet/1011302_2.png</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -5115,7 +5111,7 @@
       </c>
       <c r="V39" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/N%20Corp.%20E.G.O%20Fell%20Bullet/1011301.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/N%20Corp.%20E.G.O%20Fell%20Bullet/1011303_3.png</t>
         </is>
       </c>
       <c r="W39" t="n">
@@ -5198,7 +5194,7 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/The%20Thumb%20East%20Capo%20IIII/1051201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Double_Slash_-_Blast_%E7%88%86_Meursault_Icon.png/74px-Double_Slash_-_Blast_%E7%88%86_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
@@ -5218,7 +5214,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/The%20Thumb%20East%20Capo%20IIII/1051201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Triple_Slash_-_Blast_%E7%88%86_Meursault_Icon.png/74px-Triple_Slash_-_Blast_%E7%88%86_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -5238,7 +5234,7 @@
       </c>
       <c r="V40" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/The%20Thumb%20East%20Capo%20IIII/1051201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Tanglecleaver_%E5%BF%AB%E5%88%80%E4%BA%82%E9%BA%BB_Meursault_Icon.png/74px-Tanglecleaver_%E5%BF%AB%E5%88%80%E4%BA%82%E9%BA%BB_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="W40" t="n">
@@ -5321,7 +5317,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/The%20Thumb%20East%20Soldato%20II/1101301_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Adherence_to_Propriety._Sinclair_Icon.png/74px-Adherence_to_Propriety._Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
@@ -5341,7 +5337,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/The%20Thumb%20East%20Soldato%20II/1101301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Respect_the_Thumb._Sinclair_Icon.png/74px-Respect_the_Thumb._Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -5361,7 +5357,7 @@
       </c>
       <c r="V41" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/The%20Thumb%20East%20Soldato%20II/1101301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Thruster_Compression_Sinclair_Icon.png/74px-Thruster_Compression_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="W41" t="n">
@@ -5444,7 +5440,7 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Family%20Hierarch%20Candidate/1081201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Crimson_Strike_Ishmael_Icon.png/74px-Crimson_Strike_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
@@ -5464,7 +5460,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Family%20Hierarch%20Candidate/1081201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Crimson_Phoenix_Ishmael_Icon.png/74px-Crimson_Phoenix_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -5484,7 +5480,7 @@
       </c>
       <c r="V42" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Family%20Hierarch%20Candidate/1081201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Crimson_Spring_Ishmael_Icon.png/74px-Crimson_Spring_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="W42" t="n">
@@ -5563,7 +5559,7 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Heishou%20Pack%20-%20Mao%20Branch%20Adept/1021201_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Blinkstep_Faust_Icon.png/74px-Blinkstep_Faust_Icon.png</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
@@ -5583,7 +5579,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Heishou%20Pack%20-%20Mao%20Branch%20Adept/1021201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Clearing_the_Path%2C_My_Lord_Faust_Icon.png/74px-Clearing_the_Path%2C_My_Lord_Faust_Icon.png</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -5603,7 +5599,7 @@
       </c>
       <c r="V43" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Heishou%20Pack%20-%20Mao%20Branch%20Adept/1021201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Traceless_to_Sight_and_Sound_Alike_Faust_Icon.png/74px-Traceless_to_Sight_and_Sound_Alike_Faust_Icon.png</t>
         </is>
       </c>
       <c r="W43" t="n">
@@ -5686,7 +5682,7 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Heishou%20Pack%20-%20Si%20Branch/1091201_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Serpent_Glint_Rodion_Icon.png/74px-Serpent_Glint_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
@@ -5706,7 +5702,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Heishou%20Pack%20-%20Si%20Branch/1091201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Snake_Fang_Rodion_Icon.png/74px-Snake_Fang_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -5726,7 +5722,7 @@
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Heishou%20Pack%20-%20Si%20Branch/1091201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Serpent%27s_Mortal_Flurry_Rodion_Icon.png/74px-Serpent%27s_Mortal_Flurry_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="W44" t="n">
@@ -5829,7 +5825,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Heishou%20Pack%20-%20Si%20Branch/1121201.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Heishou%20Pack%20-%20Si%20Branch/1121202_2.png</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
@@ -5849,7 +5845,7 @@
       </c>
       <c r="V45" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Heishou%20Pack%20-%20Si%20Branch/1121201.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Heishou%20Pack%20-%20Si%20Branch/1121203_3.png</t>
         </is>
       </c>
       <c r="W45" t="n">
@@ -5932,7 +5928,7 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/R%20Corp.%204th%20Pack%20Reindeer/1061201_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Energy_Strike_Hong_Lu_Icon.png/74px-Energy_Strike_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
@@ -5952,7 +5948,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/R%20Corp.%204th%20Pack%20Reindeer/1061201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Mind_Whip_Hong_Lu_Icon.png/74px-Mind_Whip_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
@@ -5972,7 +5968,7 @@
       </c>
       <c r="V46" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/R%20Corp.%204th%20Pack%20Reindeer/1061201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Concentration_Hong_Lu_Icon.png/74px-Concentration_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="W46" t="n">
@@ -6051,7 +6047,7 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/The%20Middle%20Little%20Brother/1101201_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Is_it_You%3F%21_Sinclair_Icon.png/74px-Is_it_You%3F%21_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
@@ -6071,7 +6067,7 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/The%20Middle%20Little%20Brother/1101201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Payback_with_Interest_Sinclair_Icon.png/74px-Payback_with_Interest_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
@@ -6091,7 +6087,7 @@
       </c>
       <c r="V47" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/The%20Middle%20Little%20Brother/1101201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Write_%27em_all_down_Sinclair_Icon.png/74px-Write_%27em_all_down_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="W47" t="n">
@@ -6170,7 +6166,7 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Heishou%20Pack%20-%20Mao%20Branch/1041101_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Blinkstep_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Blinkstep_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
@@ -6190,7 +6186,7 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Heishou%20Pack%20-%20Mao%20Branch/1041101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/As_Written_Ry%C5%8Dsh%C5%AB_Icon.png/74px-As_Written_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
@@ -6210,7 +6206,7 @@
       </c>
       <c r="V48" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Heishou%20Pack%20-%20Mao%20Branch/1041101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/I%27ll_gut_you_with_a_curse-engraved_sword_Ry%C5%8Dsh%C5%AB_Icon.png/74px-I%27ll_gut_you_with_a_curse-engraved_sword_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="W48" t="n">
@@ -6289,7 +6285,7 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/Heishou%20Pack%20-%20Mao%20Branch/1111201_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Blinkstep_Outis_Icon.png/74px-Blinkstep_Outis_Icon.png</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
@@ -6309,7 +6305,7 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/Heishou%20Pack%20-%20Mao%20Branch/1111201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Perforating_Kill_Outis_Icon.png/74px-Perforating_Kill_Outis_Icon.png</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
@@ -6329,7 +6325,7 @@
       </c>
       <c r="V49" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/Heishou%20Pack%20-%20Mao%20Branch/1111201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Cursewrit_Butcherblade_Outis_Icon.png/74px-Cursewrit_Butcherblade_Outis_Icon.png</t>
         </is>
       </c>
       <c r="W49" t="n">
@@ -6412,7 +6408,7 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/Cinq%20Assoc.%20East%20Section%203/1031101_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Fa_Jin_Don_Quixote_Icon.png/74px-Fa_Jin_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
@@ -6432,7 +6428,7 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/Cinq%20Assoc.%20East%20Section%203/1031101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Virescent_Flame_Palm_Don_Quixote_Icon.png/74px-Virescent_Flame_Palm_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
@@ -6452,7 +6448,7 @@
       </c>
       <c r="V50" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/Cinq%20Assoc.%20East%20Section%203/1031101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Prithee%2C_let_this_be_an_enlightening_bout_Don_Quixote_Icon.png/74px-Prithee%2C_let_this_be_an_enlightening_bout_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="W50" t="n">
@@ -6551,7 +6547,7 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Firefist%20Office%20Survivor/1121101.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Firefist%20Office%20Survivor/1121102_2.png</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
@@ -6571,7 +6567,7 @@
       </c>
       <c r="V51" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Firefist%20Office%20Survivor/1121101.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Firefist%20Office%20Survivor/1121103_3.png</t>
         </is>
       </c>
       <c r="W51" t="n">
@@ -6650,7 +6646,7 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Liu%20Assoc.%20South%20Section%203/1011201_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Flame_Hew_Yi_Sang_Icon.png/74px-Flame_Hew_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
@@ -6670,7 +6666,7 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Liu%20Assoc.%20South%20Section%203/1011201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Frontal_Assault_Yi_Sang_Icon.png/74px-Frontal_Assault_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
@@ -6690,7 +6686,7 @@
       </c>
       <c r="V52" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Liu%20Assoc.%20South%20Section%203/1011201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Flow_of_the_Sword_Yi_Sang_Icon.png/74px-Flow_of_the_Sword_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="W52" t="n">
@@ -6769,7 +6765,7 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Kurokumo%20Clan%20Wakashu/1071201_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Lenticular_Rend_Heathcliff_Icon.png/74px-Lenticular_Rend_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
@@ -6789,7 +6785,7 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Kurokumo%20Clan%20Wakashu/1071201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Stormcloud_Heathcliff_Icon.png/74px-Stormcloud_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
@@ -6809,7 +6805,7 @@
       </c>
       <c r="V53" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Kurokumo%20Clan%20Wakashu/1071201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Thundercleave_Heathcliff_Icon.png/74px-Thundercleave_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="W53" t="n">
@@ -6888,7 +6884,7 @@
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Kurokumo%20Clan%20Captain/1081101_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Clean_Up_Ishmael_Icon.png/74px-Clean_Up_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
@@ -6908,7 +6904,7 @@
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Kurokumo%20Clan%20Captain/1081101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Sharpened_Blade_Ishmael_Icon.png/74px-Sharpened_Blade_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
@@ -6928,7 +6924,7 @@
       </c>
       <c r="V54" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Kurokumo%20Clan%20Captain/1081101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Ink_Over_Ishmael_Icon.png/74px-Ink_Over_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="W54" t="n">
@@ -7027,7 +7023,7 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/LCE%20E.G.O%20Lantern/1011101.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/LCE%20E.G.O%20Lantern/1011102_2.png</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
@@ -7047,7 +7043,7 @@
       </c>
       <c r="V55" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/LCE%20E.G.O%20Lantern/1011101.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/LCE%20E.G.O%20Lantern/1011103_3.png</t>
         </is>
       </c>
       <c r="W55" t="n">
@@ -7146,7 +7142,7 @@
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/LCE%20E.G.O%20Ardor%20Blossom%20Star/1021101.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Faust/LCE%20E.G.O%20Ardor%20Blossom%20Star/1021102_2.png</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
@@ -7166,7 +7162,7 @@
       </c>
       <c r="V56" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/LCE%20E.G.O%20Ardor%20Blossom%20Star/1021101.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Faust/LCE%20E.G.O%20Ardor%20Blossom%20Star/1021103.png</t>
         </is>
       </c>
       <c r="W56" t="n">
@@ -7245,7 +7241,7 @@
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Full-Stop%20Office%20Rep/1061101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Take_the_Shot_Hong_Lu_Icon.png/74px-Take_the_Shot_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">
@@ -7265,7 +7261,7 @@
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Full-Stop%20Office%20Rep/1061101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Target_Marked_Hong_Lu_Icon.png/74px-Target_Marked_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
@@ -7285,7 +7281,7 @@
       </c>
       <c r="V57" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Full-Stop%20Office%20Rep/1061101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Full-Stop_to_Life_Hong_Lu_Icon.png/74px-Full-Stop_to_Life_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="W57" t="n">
@@ -7364,7 +7360,7 @@
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Full-Stop%20Office%20Fixer/1071101_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Return_Fire_Heathcliff_Icon.png/74px-Return_Fire_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="O58" t="inlineStr">
@@ -7384,7 +7380,7 @@
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Full-Stop%20Office%20Fixer/1071101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Headshot_Heathcliff_Icon.png/74px-Headshot_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
@@ -7404,7 +7400,7 @@
       </c>
       <c r="V58" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Full-Stop%20Office%20Fixer/1071101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Goin%27_for_the_Bullseye_Heathcliff_Icon.png/74px-Goin%27_for_the_Bullseye_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="W58" t="n">
@@ -7483,7 +7479,7 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/The%20Manager%20of%20La%20Manchaland/1031001.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Enough_is_Enough_Don_Quixote_Icon.png/74px-Enough_is_Enough_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
@@ -7503,7 +7499,7 @@
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/The%20Manager%20of%20La%20Manchaland/1031001.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Let_All_Blossom_Free_Don_Quixote_Icon.png/74px-Let_All_Blossom_Free_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
@@ -7523,7 +7519,7 @@
       </c>
       <c r="V59" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/The%20Manager%20of%20La%20Manchaland/1031001.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/I_Shall_Impale_Don_Quixote_Icon.png/74px-I_Shall_Impale_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="W59" t="n">
@@ -7602,7 +7598,7 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Devyat_%20Assoc.%20North%20Section%203/1101101_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Courier_Trunk_-_Decay_Hammer_Sinclair_Icon.png/74px-Courier_Trunk_-_Decay_Hammer_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
@@ -7622,7 +7618,7 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Devyat_%20Assoc.%20North%20Section%203/1101101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Courier_Trunk_-_Demolition_Gadget_Sinclair_Icon.png/74px-Courier_Trunk_-_Demolition_Gadget_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
@@ -7642,7 +7638,7 @@
       </c>
       <c r="V60" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Devyat_%20Assoc.%20North%20Section%203/1101101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Poludnitsa..._I_trust_you%21_Sinclair_Icon.png/74px-Poludnitsa..._I_trust_you%21_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="W60" t="n">
@@ -7725,7 +7721,7 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/The%20Princess%20of%20La%20ManchaLand/1091101_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Begone_Rodion_Icon.png/74px-Begone_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
@@ -7745,7 +7741,7 @@
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/The%20Princess%20of%20La%20ManchaLand/1091101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/In_Finely_Ground_Mistfall_Rodion_Icon.png/74px-In_Finely_Ground_Mistfall_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
@@ -7765,7 +7761,7 @@
       </c>
       <c r="V61" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/The%20Princess%20of%20La%20ManchaLand/1091101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/The_Festival_Will_End_Rodion_Icon.png/74px-The_Festival_Will_End_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="W61" t="n">
@@ -7868,7 +7864,7 @@
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/The%20Priest%20of%20La%20Manchaland/1121001.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/The%20Priest%20of%20La%20Manchaland/1121002_2.png</t>
         </is>
       </c>
       <c r="S62" t="inlineStr">
@@ -7888,7 +7884,7 @@
       </c>
       <c r="V62" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/The%20Priest%20of%20La%20Manchaland/1121001.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/The%20Priest%20of%20La%20Manchaland/1121003_3.png</t>
         </is>
       </c>
       <c r="W62" t="n">
@@ -7967,7 +7963,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Fanghunt%20Office%20Fixer/1061001_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Slam_Hong_Lu_Icon.png/74px-Slam_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="O63" t="inlineStr">
@@ -7987,7 +7983,7 @@
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Fanghunt%20Office%20Fixer/1061001.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Bonecrusher_Hong_Lu_Icon.png/74px-Bonecrusher_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="S63" t="inlineStr">
@@ -8007,7 +8003,7 @@
       </c>
       <c r="V63" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Fanghunt%20Office%20Fixer/1061001.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/A_Cheerful_Hunt%27s_End_Hong_Lu_Icon.png/74px-A_Cheerful_Hunt%27s_End_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="W63" t="n">
@@ -8086,7 +8082,7 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/The%20Barber%20of%20La%20Manchaland/1111101_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Sewing_Outis_Icon.png/74px-Sewing_Outis_Icon.png</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
@@ -8106,7 +8102,7 @@
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/The%20Barber%20of%20La%20Manchaland/1111101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Scission_Outis_Icon.png/74px-Scission_Outis_Icon.png</t>
         </is>
       </c>
       <c r="S64" t="inlineStr">
@@ -8126,7 +8122,7 @@
       </c>
       <c r="V64" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/The%20Barber%20of%20La%20Manchaland/1111101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/I%27ll_Make_You_a_New_Dress%21_Outis_Icon.png/74px-I%27ll_Make_You_a_New_Dress%21_Outis_Icon.png</t>
         </is>
       </c>
       <c r="W64" t="n">
@@ -8209,7 +8205,7 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Cinq%20Assoc.%20West%20Section%203/1051101_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Allez_Meursault_Icon.png/74px-Allez_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
@@ -8229,7 +8225,7 @@
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Cinq%20Assoc.%20West%20Section%203/1051101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Fente_Meursault_Icon.png/74px-Fente_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">
@@ -8249,7 +8245,7 @@
       </c>
       <c r="V65" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Cinq%20Assoc.%20West%20Section%203/1051101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Salut_Meursault_Icon.png/74px-Salut_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="W65" t="n">
@@ -8328,7 +8324,7 @@
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Zwei%20Assoc.%20West%20Section%203/1101001_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Suppressing_Sinclair_Icon.png/74px-Suppressing_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="O66" t="inlineStr">
@@ -8348,7 +8344,7 @@
       </c>
       <c r="R66" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Zwei%20Assoc.%20West%20Section%203/1101001.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Combat_Preparation_Sinclair_Icon.png/74px-Combat_Preparation_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="S66" t="inlineStr">
@@ -8368,7 +8364,7 @@
       </c>
       <c r="V66" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Zwei%20Assoc.%20West%20Section%203/1101001.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Fence_Sinclair_Icon.png/74px-Fence_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="W66" t="n">
@@ -8447,7 +8443,7 @@
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Zwei%20Assoc.%20West%20Section%203/1081001_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Zwei_Knight%27s_Greatsword_Form_Ishmael_Icon.png/74px-Zwei_Knight%27s_Greatsword_Form_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
@@ -8467,7 +8463,7 @@
       </c>
       <c r="R67" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Zwei%20Assoc.%20West%20Section%203/1081001.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Can%27t_Let_You_Through_Ishmael_Icon.png/74px-Can%27t_Let_You_Through_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="S67" t="inlineStr">
@@ -8487,7 +8483,7 @@
       </c>
       <c r="V67" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Zwei%20Assoc.%20West%20Section%203/1081001.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Ward_Ishmael_Icon.png/74px-Ward_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="W67" t="n">
@@ -8566,7 +8562,7 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Devyat_%20Assoc.%20North%20Section%203/1091001_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Courier_Trunk_-_Decay_Knife_Rodion_Icon.png/74px-Courier_Trunk_-_Decay_Knife_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
@@ -8586,7 +8582,7 @@
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Devyat_%20Assoc.%20North%20Section%203/1091001.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Courier_Trunk_-_Gadget_Reveal_Rodion_Icon.png/74px-Courier_Trunk_-_Gadget_Reveal_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="S68" t="inlineStr">
@@ -8606,7 +8602,7 @@
       </c>
       <c r="V68" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Devyat_%20Assoc.%20North%20Section%203/1091001.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/I_Trust_Ya_Polu_Rodion_Icon.png/74px-I_Trust_Ya_Polu_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="W68" t="n">
@@ -8685,7 +8681,7 @@
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Lobotomy%20E.G.O%20Solemn%20Lament/1011001_1.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Lobotomy%20E.G.O%20Solemn%20Lament/1011001.png</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
@@ -8705,7 +8701,7 @@
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Lobotomy%20E.G.O%20Solemn%20Lament/1011001.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Lobotomy%20E.G.O%20Solemn%20Lament/1011002.png</t>
         </is>
       </c>
       <c r="S69" t="inlineStr">
@@ -8725,7 +8721,7 @@
       </c>
       <c r="V69" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Lobotomy%20E.G.O%20Solemn%20Lament/1011001.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Lobotomy%20E.G.O%20Solemn%20Lament/1011003.png</t>
         </is>
       </c>
       <c r="W69" t="n">
@@ -8828,7 +8824,7 @@
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Lobotomy%20E.G.O%20Red%20Eyes%20%26%20Penitence/1041001.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Lobotomy%20E.G.O%20Red%20Eyes%20%26%20Penitence/1041002_2.png</t>
         </is>
       </c>
       <c r="S70" t="inlineStr">
@@ -8848,7 +8844,7 @@
       </c>
       <c r="V70" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Lobotomy%20E.G.O%20Red%20Eyes%20%26%20Penitence/1041001.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Lobotomy%20E.G.O%20Red%20Eyes%20%26%20Penitence/1041003.png</t>
         </is>
       </c>
       <c r="W70" t="n">
@@ -8927,7 +8923,7 @@
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Wild%20Hunt/1071001_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Beheading_Heathcliff_Icon.png/74px-Beheading_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="O71" t="inlineStr">
@@ -8947,7 +8943,7 @@
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Wild%20Hunt/1071001.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Memorial_Procession_Heathcliff_Icon.png/74px-Memorial_Procession_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="S71" t="inlineStr">
@@ -8967,7 +8963,7 @@
       </c>
       <c r="V71" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Wild%20Hunt/1071001.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Requiem_Heathcliff_Icon.png/74px-Requiem_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="W71" t="n">
@@ -9046,7 +9042,7 @@
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/MultiCrack%20Office%20Rep/1021001_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/40Y-3_Activation_Faust_Icon.png/74px-40Y-3_Activation_Faust_Icon.png</t>
         </is>
       </c>
       <c r="O72" t="inlineStr">
@@ -9066,7 +9062,7 @@
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/MultiCrack%20Office%20Rep/1021001.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Charge_Countercurrent_Faust_Icon.png/74px-Charge_Countercurrent_Faust_Icon.png</t>
         </is>
       </c>
       <c r="S72" t="inlineStr">
@@ -9086,7 +9082,7 @@
       </c>
       <c r="V72" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/MultiCrack%20Office%20Rep/1021001.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/40Y-3_Charge_Faust_Icon.png/74px-40Y-3_Charge_Faust_Icon.png</t>
         </is>
       </c>
       <c r="W72" t="n">
@@ -9165,7 +9161,7 @@
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/MultiCrack%20Office%20Fixer/1070901_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/40S-2_Activation_Heathcliff_Icon.png/74px-40S-2_Activation_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="O73" t="inlineStr">
@@ -9185,7 +9181,7 @@
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/MultiCrack%20Office%20Fixer/1070901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Photoelectric_Mark_Heathcliff_Icon.png/74px-Photoelectric_Mark_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="S73" t="inlineStr">
@@ -9205,7 +9201,7 @@
       </c>
       <c r="V73" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/MultiCrack%20Office%20Fixer/1070901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Photoelectric_Harpoon_Heathcliff_Icon.png/74px-Photoelectric_Harpoon_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="W73" t="n">
@@ -9288,7 +9284,7 @@
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/W%20Corp.%20L3%20Cleanup%20Captain/1111001_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Ripple_Outis_Icon.png/74px-Ripple_Outis_Icon.png</t>
         </is>
       </c>
       <c r="O74" t="inlineStr">
@@ -9308,7 +9304,7 @@
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/W%20Corp.%20L3%20Cleanup%20Captain/1111001.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Charged_Leap_Outis_Icon.png/74px-Charged_Leap_Outis_Icon.png</t>
         </is>
       </c>
       <c r="S74" t="inlineStr">
@@ -9328,7 +9324,7 @@
       </c>
       <c r="V74" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/W%20Corp.%20L3%20Cleanup%20Captain/1111001.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Rip_Dimension_Outis_Icon.png/74px-Rip_Dimension_Outis_Icon.png</t>
         </is>
       </c>
       <c r="W74" t="n">
@@ -9407,7 +9403,7 @@
       </c>
       <c r="N75" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Dieci%20Assoc.%20South%20Section%204%20Director/1051001_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Studious_Dedication_Meursault_Icon.png/74px-Studious_Dedication_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="O75" t="inlineStr">
@@ -9427,7 +9423,7 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Dieci%20Assoc.%20South%20Section%204%20Director/1051001.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Moment_of_Erudition_Meursault_Icon.png/74px-Moment_of_Erudition_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
@@ -9447,7 +9443,7 @@
       </c>
       <c r="V75" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Dieci%20Assoc.%20South%20Section%204%20Director/1051001.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Scorch_Knowledge_Meursault_Icon.png/74px-Scorch_Knowledge_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="W75" t="n">
@@ -9526,7 +9522,7 @@
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/T%20Corp.%20Class%203%20Collection%20Staff/1030901_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Let_Us_Prepare_to_Collect_Don_Quixote_Skill.png/74px-Let_Us_Prepare_to_Collect_Don_Quixote_Skill.png</t>
         </is>
       </c>
       <c r="O76" t="inlineStr">
@@ -9546,7 +9542,7 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/T%20Corp.%20Class%203%20Collection%20Staff/1030901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/T_Corp._Accelerated_Amputator_Don_Quixote_Skill.png/74px-T_Corp._Accelerated_Amputator_Don_Quixote_Skill.png</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
@@ -9566,7 +9562,7 @@
       </c>
       <c r="V76" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/T%20Corp.%20Class%203%20Collection%20Staff/1030901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/I_Command_Thee_Halt_Don_Quixote_Skill.png/74px-I_Command_Thee_Halt_Don_Quixote_Skill.png</t>
         </is>
       </c>
       <c r="W76" t="n">
@@ -9645,7 +9641,7 @@
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/T%20Corp.%20Class%202%20Collection%20Staff/1090901_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Prepare_to_Collect_Rodion_Skill.png/74px-Prepare_to_Collect_Rodion_Skill.png</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
@@ -9665,7 +9661,7 @@
       </c>
       <c r="R77" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/T%20Corp.%20Class%202%20Collection%20Staff/1090901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/T_Corp._Martial_Suppression_Rodion_Skill.png/74px-T_Corp._Martial_Suppression_Rodion_Skill.png</t>
         </is>
       </c>
       <c r="S77" t="inlineStr">
@@ -9685,7 +9681,7 @@
       </c>
       <c r="V77" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/T%20Corp.%20Class%202%20Collection%20Staff/1090901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Execute_Collections_Rodion_Skill.png/74px-Execute_Collections_Rodion_Skill.png</t>
         </is>
       </c>
       <c r="W77" t="n">
@@ -9764,7 +9760,7 @@
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/District%2020%20Yurodivy/1040901_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Got_a_Screw_Loose_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Got_a_Screw_Loose_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="O78" t="inlineStr">
@@ -9784,7 +9780,7 @@
       </c>
       <c r="R78" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/District%2020%20Yurodivy/1040901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Compression_Wind-up_Spanner_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Compression_Wind-up_Spanner_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="S78" t="inlineStr">
@@ -9804,7 +9800,7 @@
       </c>
       <c r="V78" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/District%2020%20Yurodivy/1040901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Percussive_Maintenance_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Percussive_Maintenance_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="W78" t="n">
@@ -9883,7 +9879,7 @@
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/District%2020%20Yurodivy/1060901_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Deduction_Start_Hong_Lu_Icon.png/74px-Deduction_Start_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="O79" t="inlineStr">
@@ -9903,7 +9899,7 @@
       </c>
       <c r="R79" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/District%2020%20Yurodivy/1060901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Morph_Cane_Technique_Hong_Lu_Icon.png/74px-Morph_Cane_Technique_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="S79" t="inlineStr">
@@ -9923,7 +9919,7 @@
       </c>
       <c r="V79" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/District%2020%20Yurodivy/1060901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/You%27re_the_Culprit_Hong_Lu_Icon.png/74px-You%27re_the_Culprit_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="W79" t="n">
@@ -10002,7 +9998,7 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/The%20Ring%20Pointillist%20Student/1010901_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Paint_Over_Yi_Sang_Icon.png/74px-Paint_Over_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
@@ -10022,7 +10018,7 @@
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/The%20Ring%20Pointillist%20Student/1010901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Sanguine_Pointillism_Yi_Sang_Icon.png/74px-Sanguine_Pointillism_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="S80" t="inlineStr">
@@ -10042,7 +10038,7 @@
       </c>
       <c r="V80" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/The%20Ring%20Pointillist%20Student/1010901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Hematic_Coloring_Yi_Sang_Icon.png/74px-Hematic_Coloring_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="W80" t="n">
@@ -10121,7 +10117,7 @@
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/The%20Ring%20Pointillist%20Student/1110901_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Dotting_Outis_Icon.png/74px-Dotting_Outis_Icon.png</t>
         </is>
       </c>
       <c r="O81" t="inlineStr">
@@ -10141,7 +10137,7 @@
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/The%20Ring%20Pointillist%20Student/1110901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Sanguine_Painting_Outis_Icon.png/74px-Sanguine_Painting_Outis_Icon.png</t>
         </is>
       </c>
       <c r="S81" t="inlineStr">
@@ -10161,7 +10157,7 @@
       </c>
       <c r="V81" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/The%20Ring%20Pointillist%20Student/1110901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Artwork_Inspection_Outis_Icon.png/74px-Artwork_Inspection_Outis_Icon.png</t>
         </is>
       </c>
       <c r="W81" t="n">
@@ -10240,7 +10236,7 @@
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Dawn%20Office%20Fixer/1100901_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Fierce_Charge_Sinclair_Icon.png/74px-Fierce_Charge_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="O82" t="inlineStr">
@@ -10260,7 +10256,7 @@
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Dawn%20Office%20Fixer/1100901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Sunset_Blade_Sinclair_Icon.png/74px-Sunset_Blade_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="S82" t="inlineStr">
@@ -10280,7 +10276,7 @@
       </c>
       <c r="V82" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Dawn%20Office%20Fixer/1100901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Stigmatize_Sinclair_Icon.png/74px-Stigmatize_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="W82" t="n">
@@ -10359,7 +10355,7 @@
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Edgar%20Family%20Chief%20Butler/1040801_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Receiving_Arts_1_The_Hunt_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Receiving_Arts_1_The_Hunt_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="O83" t="inlineStr">
@@ -10379,7 +10375,7 @@
       </c>
       <c r="R83" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Edgar%20Family%20Chief%20Butler/1040801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Receiving_Arts_7_Capture_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Receiving_Arts_7_Capture_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="S83" t="inlineStr">
@@ -10399,7 +10395,7 @@
       </c>
       <c r="V83" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Edgar%20Family%20Chief%20Butler/1040801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Receiving_Arts_2_S.Y.N.C._Ry%C5%8Dsh%C5%AB_Icon.png/74px-Receiving_Arts_2_S.Y.N.C._Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="W83" t="n">
@@ -10482,7 +10478,7 @@
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Edgar%20Family%20Butler/1080901_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Sweeping_Redirection_Ishmael_Icon.png/74px-Sweeping_Redirection_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="O84" t="inlineStr">
@@ -10502,7 +10498,7 @@
       </c>
       <c r="R84" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Edgar%20Family%20Butler/1080901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Housekeeping_Ishmael_Icon.png/74px-Housekeeping_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="S84" t="inlineStr">
@@ -10522,7 +10518,7 @@
       </c>
       <c r="V84" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Edgar%20Family%20Butler/1080901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Restraining_Technique_Ishmael_Icon.png/74px-Restraining_Technique_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="W84" t="n">
@@ -10601,7 +10597,7 @@
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Wuthering%20Heights%20Butler/1020901_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Confiscation_Faust_Icon.png/74px-Confiscation_Faust_Icon.png</t>
         </is>
       </c>
       <c r="O85" t="inlineStr">
@@ -10621,7 +10617,7 @@
       </c>
       <c r="R85" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Wuthering%20Heights%20Butler/1020901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Interloper_Reception_Faust_Icon.png/74px-Interloper_Reception_Faust_Icon.png</t>
         </is>
       </c>
       <c r="S85" t="inlineStr">
@@ -10641,7 +10637,7 @@
       </c>
       <c r="V85" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Wuthering%20Heights%20Butler/1020901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Reception_Arts_4_Heartseal_Faust_Icon.png/74px-Reception_Arts_4_Heartseal_Faust_Icon.png</t>
         </is>
       </c>
       <c r="W85" t="n">
@@ -10740,7 +10736,7 @@
       </c>
       <c r="R86" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Edgar%20Family%20Heir/1120901.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Edgar%20Family%20Heir/1120902_2.png</t>
         </is>
       </c>
       <c r="S86" t="inlineStr">
@@ -10760,7 +10756,7 @@
       </c>
       <c r="V86" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Edgar%20Family%20Heir/1120901.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Edgar%20Family%20Heir/1120903_3.png</t>
         </is>
       </c>
       <c r="W86" t="n">
@@ -10839,7 +10835,7 @@
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Dead%20Rabbits%20Boss/1050901_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Bat_Strike_Meursault_Icon.png/74px-Bat_Strike_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="O87" t="inlineStr">
@@ -10859,7 +10855,7 @@
       </c>
       <c r="R87" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Dead%20Rabbits%20Boss/1050901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Smackdown_Meursault_Icon.png/74px-Smackdown_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="S87" t="inlineStr">
@@ -10879,7 +10875,7 @@
       </c>
       <c r="V87" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Dead%20Rabbits%20Boss/1050901.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Relentless_Meursault_Icon.png/74px-Relentless_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="W87" t="n">
@@ -10958,7 +10954,7 @@
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/Wuthering%20Heights%20Chief%20Butler/1110801_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Knocking_Outis_Icon.png/74px-Knocking_Outis_Icon.png</t>
         </is>
       </c>
       <c r="O88" t="inlineStr">
@@ -10978,7 +10974,7 @@
       </c>
       <c r="R88" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/Wuthering%20Heights%20Chief%20Butler/1110801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Dusting_Outis_Icon.png/74px-Dusting_Outis_Icon.png</t>
         </is>
       </c>
       <c r="S88" t="inlineStr">
@@ -10998,7 +10994,7 @@
       </c>
       <c r="V88" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/Wuthering%20Heights%20Chief%20Butler/1110801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/As_Mistress_Commands_Outis_Icon.png/74px-As_Mistress_Commands_Outis_Icon.png</t>
         </is>
       </c>
       <c r="W88" t="n">
@@ -11077,7 +11073,7 @@
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Oufi%20Assoc.%20South%20Section%203/1070801_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Execution_Advised_Heathcliff_Icon.png/74px-Execution_Advised_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="O89" t="inlineStr">
@@ -11097,7 +11093,7 @@
       </c>
       <c r="R89" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Oufi%20Assoc.%20South%20Section%203/1070801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Final_Warning_Heathcliff_Icon.png/74px-Final_Warning_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="S89" t="inlineStr">
@@ -11117,7 +11113,7 @@
       </c>
       <c r="V89" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Oufi%20Assoc.%20South%20Section%203/1070801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Execution_Sentencing_Heathcliff_Icon.png/74px-Execution_Sentencing_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="W89" t="n">
@@ -11196,7 +11192,7 @@
       </c>
       <c r="N90" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Liu%20Assoc.%20South%20Section%204/1040701_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/All-out_War_Ry%C5%8Dsh%C5%AB_Icon.png/74px-All-out_War_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="O90" t="inlineStr">
@@ -11216,7 +11212,7 @@
       </c>
       <c r="R90" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Liu%20Assoc.%20South%20Section%204/1040701.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Fiery_Knifehand_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Fiery_Knifehand_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="S90" t="inlineStr">
@@ -11236,7 +11232,7 @@
       </c>
       <c r="V90" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Liu%20Assoc.%20South%20Section%204/1040701.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Flame_Cleave_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Flame_Cleave_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="W90" t="n">
@@ -11315,7 +11311,7 @@
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Liu%20Assoc.%20South%20Section%204%20Director/1090801_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Flaming_Fists_Rodion_Icon.png/74px-Flaming_Fists_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="O91" t="inlineStr">
@@ -11335,7 +11331,7 @@
       </c>
       <c r="R91" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Liu%20Assoc.%20South%20Section%204%20Director/1090801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Fiery_Knifehand-Combust_Rodion_Icon.png/74px-Fiery_Knifehand-Combust_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="S91" t="inlineStr">
@@ -11355,7 +11351,7 @@
       </c>
       <c r="V91" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Liu%20Assoc.%20South%20Section%204%20Director/1090801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Pinpoint_Blitz_Rodion_Icon.png/74px-Pinpoint_Blitz_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="W91" t="n">
@@ -11434,7 +11430,7 @@
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Blade%20Lineage%20Salsu/1020801_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Moonlit_Blade_Dance_Faust_Icon.png/74px-Moonlit_Blade_Dance_Faust_Icon.png</t>
         </is>
       </c>
       <c r="O92" t="inlineStr">
@@ -11454,7 +11450,7 @@
       </c>
       <c r="R92" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Blade%20Lineage%20Salsu/1020801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Acupuncture_Faust_Icon.png/74px-Acupuncture_Faust_Icon.png</t>
         </is>
       </c>
       <c r="S92" t="inlineStr">
@@ -11474,7 +11470,7 @@
       </c>
       <c r="V92" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Blade%20Lineage%20Salsu/1020801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Red_Plum_Blossoms_Scatter_Faust_Icon.png/74px-Red_Plum_Blossoms_Scatter_Faust_Icon.png</t>
         </is>
       </c>
       <c r="W92" t="n">
@@ -11553,7 +11549,7 @@
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/Blade%20Lineage%20Salsu/1030801_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Draw_of_the_Sword_Don_Quixote_Icon.png/74px-Draw_of_the_Sword_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="O93" t="inlineStr">
@@ -11573,7 +11569,7 @@
       </c>
       <c r="R93" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/Blade%20Lineage%20Salsu/1030801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Blade_Arc_Don_Quixote_Icon.png/74px-Blade_Arc_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="S93" t="inlineStr">
@@ -11593,7 +11589,7 @@
       </c>
       <c r="V93" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/Blade%20Lineage%20Salsu/1030801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Fare_Thee_Well_Don_Quixote_Icon.png/74px-Fare_Thee_Well_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="W93" t="n">
@@ -11672,7 +11668,7 @@
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Blade%20Lineage%20Mentor/1050801_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Draw_of_the_Sword_Meursault_Icon.png/74px-Draw_of_the_Sword_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="O94" t="inlineStr">
@@ -11692,7 +11688,7 @@
       </c>
       <c r="R94" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Blade%20Lineage%20Mentor/1050801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Acupuncture_Meursault_Icon.png/74px-Acupuncture_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="S94" t="inlineStr">
@@ -11712,7 +11708,7 @@
       </c>
       <c r="V94" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Blade%20Lineage%20Mentor/1050801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Yield_My_Flesh_Meursault_Icon.png/74px-Yield_My_Flesh_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="W94" t="n">
@@ -11811,7 +11807,7 @@
       </c>
       <c r="R95" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Kurokumo%20Clan%20Captain/1120801.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Kurokumo%20Clan%20Captain/1120802_2.png</t>
         </is>
       </c>
       <c r="S95" t="inlineStr">
@@ -11831,7 +11827,7 @@
       </c>
       <c r="V95" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Kurokumo%20Clan%20Captain/1120801.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Kurokumo%20Clan%20Captain/1120803_3.png</t>
         </is>
       </c>
       <c r="W95" t="n">
@@ -11918,7 +11914,7 @@
       </c>
       <c r="N96" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/The%20Pequod%20Captain/1080801_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/To_Me_Ishmael_Icon.png/74px-To_Me_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="O96" t="inlineStr">
@@ -11938,7 +11934,7 @@
       </c>
       <c r="R96" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/The%20Pequod%20Captain/1080801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Pursue_Them_to_the_End_Ishmael_Icon.png/74px-Pursue_Them_to_the_End_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="S96" t="inlineStr">
@@ -11958,7 +11954,7 @@
       </c>
       <c r="V96" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/The%20Pequod%20Captain/1080801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Harpoon_of_Obsession_Ishmael_Icon.png/74px-Harpoon_of_Obsession_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="W96" t="n">
@@ -12037,7 +12033,7 @@
       </c>
       <c r="N97" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Dieci%20Assoc.%20South%20Section%204/1010801_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Expend_Knowledge_Yi_Sang_Icon.png/74px-Expend_Knowledge_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="O97" t="inlineStr">
@@ -12057,7 +12053,7 @@
       </c>
       <c r="R97" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Dieci%20Assoc.%20South%20Section%204/1010801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Seal_Shut_Yi_Sang_Icon.png/74px-Seal_Shut_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="S97" t="inlineStr">
@@ -12077,7 +12073,7 @@
       </c>
       <c r="V97" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Dieci%20Assoc.%20South%20Section%204/1010801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Grace_of_Knowledge_Yi_Sang_Icon.png/74px-Grace_of_Knowledge_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="W97" t="n">
@@ -12156,7 +12152,7 @@
       </c>
       <c r="N98" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Dieci%20Assoc.%20South%20Section%204/1060801_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Expend_Knowledge_Hong_Lu_Icon.png/74px-Expend_Knowledge_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="O98" t="inlineStr">
@@ -12176,7 +12172,7 @@
       </c>
       <c r="R98" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Dieci%20Assoc.%20South%20Section%204/1060801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Unveil_Hong_Lu_Icon.png/74px-Unveil_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="S98" t="inlineStr">
@@ -12196,7 +12192,7 @@
       </c>
       <c r="V98" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Dieci%20Assoc.%20South%20Section%204/1060801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Cyclical_Knowledge_Hong_Lu_Icon.png/74px-Cyclical_Knowledge_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="W98" t="n">
@@ -12295,7 +12291,7 @@
       </c>
       <c r="R99" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/Lobotomy%20E.G.O%20Lantern/1030701.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/Lobotomy%20E.G.O%20Lantern/1030702_2.png</t>
         </is>
       </c>
       <c r="S99" t="inlineStr">
@@ -12315,7 +12311,7 @@
       </c>
       <c r="V99" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/Lobotomy%20E.G.O%20Lantern/1030701.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/Lobotomy%20E.G.O%20Lantern/1030703_3.png</t>
         </is>
       </c>
       <c r="W99" t="n">
@@ -12414,7 +12410,7 @@
       </c>
       <c r="R100" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/Lobotomy%20E.G.O%20Magic%20Bullet/1110701.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Outis/Lobotomy%20E.G.O%20Magic%20Bullet/1110702_2.png</t>
         </is>
       </c>
       <c r="S100" t="inlineStr">
@@ -12434,7 +12430,7 @@
       </c>
       <c r="V100" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/Lobotomy%20E.G.O%20Magic%20Bullet/1110701.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Outis/Lobotomy%20E.G.O%20Magic%20Bullet/1110703_3.png</t>
         </is>
       </c>
       <c r="W100" t="n">
@@ -12513,7 +12509,7 @@
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Cinq%20Assoc.%20South%20Section%204%20Director/1100801_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Remise_Sinclair_Icon.png/74px-Remise_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="O101" t="inlineStr">
@@ -12533,7 +12529,7 @@
       </c>
       <c r="R101" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Cinq%20Assoc.%20South%20Section%204%20Director/1100801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Engagement_Sinclair_Icon.png/74px-Engagement_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="S101" t="inlineStr">
@@ -12553,7 +12549,7 @@
       </c>
       <c r="V101" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Cinq%20Assoc.%20South%20Section%204%20Director/1100801.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Contre_Attaque_Sinclair_Icon.png/74px-Contre_Attaque_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="W101" t="n">
@@ -12632,7 +12628,7 @@
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/Cinq%20Assoc.%20South%20Section%204/1110601_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Marche_Outis_Icon.png/74px-Marche_Outis_Icon.png</t>
         </is>
       </c>
       <c r="O102" t="inlineStr">
@@ -12652,7 +12648,7 @@
       </c>
       <c r="R102" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/Cinq%20Assoc.%20South%20Section%204/1110601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Punition_Outis_Icon.png/74px-Punition_Outis_Icon.png</t>
         </is>
       </c>
       <c r="S102" t="inlineStr">
@@ -12672,7 +12668,7 @@
       </c>
       <c r="V102" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/Cinq%20Assoc.%20South%20Section%204/1110601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Balestra_Fente_Outis_Icon.png/74px-Balestra_Fente_Outis_Icon.png</t>
         </is>
       </c>
       <c r="W102" t="n">
@@ -12755,7 +12751,7 @@
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/The%20Pequod%20First%20Mate/1010701_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Impale_Yi_Sang_Icon.png/74px-Impale_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="O103" t="inlineStr">
@@ -12775,7 +12771,7 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/The%20Pequod%20First%20Mate/1010701.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Relentless_Stabbing_Yi_Sang_Icon.png/74px-Relentless_Stabbing_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
@@ -12795,7 +12791,7 @@
       </c>
       <c r="V103" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/The%20Pequod%20First%20Mate/1010701.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Ambush_Yi_Sang_Icon.png/74px-Ambush_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="W103" t="n">
@@ -12878,7 +12874,7 @@
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/The%20Pequod%20Harpooneer/1070701.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Stalk_Prey_Heathcliff_Icon.png/74px-Stalk_Prey_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="O104" t="inlineStr">
@@ -12898,7 +12894,7 @@
       </c>
       <c r="R104" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/The%20Pequod%20Harpooneer/1070701.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Snagharpoon_Heathcliff_Icon.png/74px-Snagharpoon_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="S104" t="inlineStr">
@@ -12918,7 +12914,7 @@
       </c>
       <c r="V104" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/The%20Pequod%20Harpooneer/1070701.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Sever_Knot_Heathcliff_Icon.png/74px-Sever_Knot_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="W104" t="n">
@@ -12997,7 +12993,7 @@
       </c>
       <c r="N105" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/The%20Middle%20Little%20Sister/1030601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Checking_the_Book_Don_Quixote_Skill.png/74px-Checking_the_Book_Don_Quixote_Skill.png</t>
         </is>
       </c>
       <c r="O105" t="inlineStr">
@@ -13017,7 +13013,7 @@
       </c>
       <c r="R105" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/The%20Middle%20Little%20Sister/1030601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Proof_of_Loyalty_Don_Quixote_Skill.png/74px-Proof_of_Loyalty_Don_Quixote_Skill.png</t>
         </is>
       </c>
       <c r="S105" t="inlineStr">
@@ -13037,7 +13033,7 @@
       </c>
       <c r="V105" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/The%20Middle%20Little%20Sister/1030601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/A_Just_Vengeance_Don_Quixote_Skill.png/74px-A_Just_Vengeance_Don_Quixote_Skill.png</t>
         </is>
       </c>
       <c r="W105" t="n">
@@ -13116,7 +13112,7 @@
       </c>
       <c r="N106" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/The%20Middle%20Little%20Brother/1050701_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/We_Remember_Meursault_Skill.png/74px-We_Remember_Meursault_Skill.png</t>
         </is>
       </c>
       <c r="O106" t="inlineStr">
@@ -13136,7 +13132,7 @@
       </c>
       <c r="R106" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/The%20Middle%20Little%20Brother/1050701.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Chains_of_Loyalty_Meursault_Skill.png/74px-Chains_of_Loyalty_Meursault_Skill.png</t>
         </is>
       </c>
       <c r="S106" t="inlineStr">
@@ -13156,7 +13152,7 @@
       </c>
       <c r="V106" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/The%20Middle%20Little%20Brother/1050701.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Recording_Meursault_Skill.png/74px-Recording_Meursault_Skill.png</t>
         </is>
       </c>
       <c r="W106" t="n">
@@ -13243,7 +13239,7 @@
       </c>
       <c r="N107" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/LCCB%20Assistant%20Manager/1040601_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Shove_Ry%C5%8Dsh%C5%AB_Skill.png/74px-Shove_Ry%C5%8Dsh%C5%AB_Skill.png</t>
         </is>
       </c>
       <c r="O107" t="inlineStr">
@@ -13263,7 +13259,7 @@
       </c>
       <c r="R107" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/LCCB%20Assistant%20Manager/1040601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/T.N._Ry%C5%8Dsh%C5%AB_Skill.png/74px-T.N._Ry%C5%8Dsh%C5%AB_Skill.png</t>
         </is>
       </c>
       <c r="S107" t="inlineStr">
@@ -13283,7 +13279,7 @@
       </c>
       <c r="V107" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/LCCB%20Assistant%20Manager/1040601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/O.O.F._Ry%C5%8Dsh%C5%AB_Skill.png/74px-O.O.F._Ry%C5%8Dsh%C5%AB_Skill.png</t>
         </is>
       </c>
       <c r="W107" t="n">
@@ -13366,7 +13362,7 @@
       </c>
       <c r="N108" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Twinhook%20Pirates%20First%20Mate/1120701.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Twinhook%20Pirates%20First%20Mate/1120701_1.png</t>
         </is>
       </c>
       <c r="O108" t="inlineStr">
@@ -13386,7 +13382,7 @@
       </c>
       <c r="R108" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Twinhook%20Pirates%20First%20Mate/1120701.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Twinhook%20Pirates%20First%20Mate/1120702_2.png</t>
         </is>
       </c>
       <c r="S108" t="inlineStr">
@@ -13406,7 +13402,7 @@
       </c>
       <c r="V108" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Twinhook%20Pirates%20First%20Mate/1120701.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Twinhook%20Pirates%20First%20Mate/1120703_3.png</t>
         </is>
       </c>
       <c r="W108" t="n">
@@ -13489,7 +13485,7 @@
       </c>
       <c r="N109" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/W%20Corp.%20L3%20Cleanup%20Agent/1010601_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Dimensional_Slit_Yi_Sang_Skill.png/74px-Dimensional_Slit_Yi_Sang_Skill.png</t>
         </is>
       </c>
       <c r="O109" t="inlineStr">
@@ -13509,7 +13505,7 @@
       </c>
       <c r="R109" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/W%20Corp.%20L3%20Cleanup%20Agent/1010601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Energy_Cycle_Yi_Sang_Skill.png/74px-Energy_Cycle_Yi_Sang_Skill.png</t>
         </is>
       </c>
       <c r="S109" t="inlineStr">
@@ -13529,7 +13525,7 @@
       </c>
       <c r="V109" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/W%20Corp.%20L3%20Cleanup%20Agent/1010601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Dimensional_Rift_Yi_Sang_Skill.png/74px-Dimensional_Rift_Yi_Sang_Skill.png</t>
         </is>
       </c>
       <c r="W109" t="n">
@@ -13608,7 +13604,7 @@
       </c>
       <c r="N110" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Lobotomy%20E.G.O%20Regret/1020701.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Faust/Lobotomy%20E.G.O%20Regret/1020701_1.png</t>
         </is>
       </c>
       <c r="O110" t="inlineStr">
@@ -13628,7 +13624,7 @@
       </c>
       <c r="R110" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Lobotomy%20E.G.O%20Regret/1020701.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Faust/Lobotomy%20E.G.O%20Regret/1020702_2.png</t>
         </is>
       </c>
       <c r="S110" t="inlineStr">
@@ -13648,7 +13644,7 @@
       </c>
       <c r="V110" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Lobotomy%20E.G.O%20Regret/1020701.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Faust/Lobotomy%20E.G.O%20Regret/1020703_3.png</t>
         </is>
       </c>
       <c r="W110" t="n">
@@ -13727,7 +13723,7 @@
       </c>
       <c r="N111" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Hook%20Office%20Fixer/1060701_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Track_Hong_Lu_Icon.png/74px-Track_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="O111" t="inlineStr">
@@ -13747,7 +13743,7 @@
       </c>
       <c r="R111" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Hook%20Office%20Fixer/1060701.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Goin%27_First_Hong_Lu_Icon.png/74px-Goin%27_First_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="S111" t="inlineStr">
@@ -13767,7 +13763,7 @@
       </c>
       <c r="V111" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Hook%20Office%20Fixer/1060701.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Rampage_Hong_Lu_Icon.png/74px-Rampage_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="W111" t="n">
@@ -13846,7 +13842,7 @@
       </c>
       <c r="N112" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Dieci%20Assoc.%20South%20Section%204/1090701_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Illuminate_Thy_Vacuity_Rodion.png/74px-Illuminate_Thy_Vacuity_Rodion.png</t>
         </is>
       </c>
       <c r="O112" t="inlineStr">
@@ -13866,7 +13862,7 @@
       </c>
       <c r="R112" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Dieci%20Assoc.%20South%20Section%204/1090701.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Weight_of_Knowledge_Rodion.png/74px-Weight_of_Knowledge_Rodion.png</t>
         </is>
       </c>
       <c r="S112" t="inlineStr">
@@ -13886,7 +13882,7 @@
       </c>
       <c r="V112" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Dieci%20Assoc.%20South%20Section%204/1090701.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Excruciating_Study_Rodion.png/74px-Excruciating_Study_Rodion.png</t>
         </is>
       </c>
       <c r="W112" t="n">
@@ -13965,7 +13961,7 @@
       </c>
       <c r="N113" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Molar%20Office%20Fixer/1010501_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Stay_Calm_Yi_Sang_Skill.png/74px-Stay_Calm_Yi_Sang_Skill.png</t>
         </is>
       </c>
       <c r="O113" t="inlineStr">
@@ -13985,7 +13981,7 @@
       </c>
       <c r="R113" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Molar%20Office%20Fixer/1010501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Gamble_Yi_Sang_Skill.png/74px-Gamble_Yi_Sang_Skill.png</t>
         </is>
       </c>
       <c r="S113" t="inlineStr">
@@ -14005,7 +14001,7 @@
       </c>
       <c r="V113" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Molar%20Office%20Fixer/1010501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Grinding_the_Molars_Yi_Sang_Skill.png/74px-Grinding_the_Molars_Yi_Sang_Skill.png</t>
         </is>
       </c>
       <c r="W113" t="n">
@@ -14084,7 +14080,7 @@
       </c>
       <c r="N114" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/Molar%20Office%20Fixer/1110501_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Wait_Up_Outis_Icon.png/74px-Wait_Up_Outis_Icon.png</t>
         </is>
       </c>
       <c r="O114" t="inlineStr">
@@ -14104,7 +14100,7 @@
       </c>
       <c r="R114" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/Molar%20Office%20Fixer/1110501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Slice_Molar_Outis_Icon.png/74px-Slice_Molar_Outis_Icon.png</t>
         </is>
       </c>
       <c r="S114" t="inlineStr">
@@ -14124,7 +14120,7 @@
       </c>
       <c r="V114" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/Molar%20Office%20Fixer/1110501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Daring_Decision_Outis_Icon.png/74px-Daring_Decision_Outis_Icon.png</t>
         </is>
       </c>
       <c r="W114" t="n">
@@ -14203,7 +14199,7 @@
       </c>
       <c r="N115" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Seven%20Assoc.%20South%20Section%204/1020601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Predictive_Analysis_Faust_Icon.png/74px-Predictive_Analysis_Faust_Icon.png</t>
         </is>
       </c>
       <c r="O115" t="inlineStr">
@@ -14223,7 +14219,7 @@
       </c>
       <c r="R115" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Seven%20Assoc.%20South%20Section%204/1020601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Dissect_Target_Faust_Icon.png/74px-Dissect_Target_Faust_Icon.png</t>
         </is>
       </c>
       <c r="S115" t="inlineStr">
@@ -14243,7 +14239,7 @@
       </c>
       <c r="V115" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Seven%20Assoc.%20South%20Section%204/1020601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Profiling_Faust_Icon.png/74px-Profiling_Faust_Icon.png</t>
         </is>
       </c>
       <c r="W115" t="n">
@@ -14322,7 +14318,7 @@
       </c>
       <c r="N116" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Seven%20Assoc.%20South%20Section%204/1070601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Intuition_Heathcliff_Icon.png/74px-Intuition_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="O116" t="inlineStr">
@@ -14342,7 +14338,7 @@
       </c>
       <c r="R116" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Seven%20Assoc.%20South%20Section%204/1070601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/The_Wrap-Up_Heathcliff_Icon.png/74px-The_Wrap-Up_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="S116" t="inlineStr">
@@ -14362,7 +14358,7 @@
       </c>
       <c r="V116" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Seven%20Assoc.%20South%20Section%204/1070601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Forensics_Heathcliff_Icon.png/74px-Forensics_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="W116" t="n">
@@ -14441,7 +14437,7 @@
       </c>
       <c r="N117" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/W%20Corp.%20L3%20Cleanup%20Agent/1040501_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/E.C._Ry%C5%8Dsh%C5%AB_Skill.png/74px-E.C._Ry%C5%8Dsh%C5%AB_Skill.png</t>
         </is>
       </c>
       <c r="O117" t="inlineStr">
@@ -14461,7 +14457,7 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/W%20Corp.%20L3%20Cleanup%20Agent/1040501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Leap_Ry%C5%8Dsh%C5%AB_Skill.png/74px-Leap_Ry%C5%8Dsh%C5%AB_Skill.png</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
@@ -14481,7 +14477,7 @@
       </c>
       <c r="V117" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/W%20Corp.%20L3%20Cleanup%20Agent/1040501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/D.D.E.D.R._Ry%C5%8Dsh%C5%AB_Skill.png/74px-D.D.E.D.R._Ry%C5%8Dsh%C5%AB_Skill.png</t>
         </is>
       </c>
       <c r="W117" t="n">
@@ -14564,7 +14560,7 @@
       </c>
       <c r="N118" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/W%20Corp.%20L2%20Cleanup%20Agent/1060601_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Energy_Cycle_Hong_Lu_Skill.png/74px-Energy_Cycle_Hong_Lu_Skill.png</t>
         </is>
       </c>
       <c r="O118" t="inlineStr">
@@ -14584,7 +14580,7 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/W%20Corp.%20L2%20Cleanup%20Agent/1060601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Cleanup_Support_Hong_Lu_Skill.png/74px-Cleanup_Support_Hong_Lu_Skill.png</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
@@ -14604,7 +14600,7 @@
       </c>
       <c r="V118" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/W%20Corp.%20L2%20Cleanup%20Agent/1060601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Deploy_Charge_Barrier_Hong_Lu_Skill.png/74px-Deploy_Charge_Barrier_Hong_Lu_Skill.png</t>
         </is>
       </c>
       <c r="W118" t="n">
@@ -14679,7 +14675,7 @@
       </c>
       <c r="N119" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Zwei%20Assoc.%20South%20Section%204/1020501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Zwei_Association_South_Section_4_Faust_Patrolling_Icon.png/74px-Zwei_Association_South_Section_4_Faust_Patrolling_Icon.png</t>
         </is>
       </c>
       <c r="O119" t="inlineStr">
@@ -14699,7 +14695,7 @@
       </c>
       <c r="R119" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Zwei%20Assoc.%20South%20Section%204/1020501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Zwei_Association_South_Section_4_Faust_Client_Protection_Icon.png/74px-Zwei_Association_South_Section_4_Faust_Client_Protection_Icon.png</t>
         </is>
       </c>
       <c r="S119" t="inlineStr">
@@ -14719,7 +14715,7 @@
       </c>
       <c r="V119" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/Zwei%20Assoc.%20South%20Section%204/1020501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Zwei_Association_South_Section_4_Faust_Law_and_Order_Icon.png/74px-Zwei_Association_South_Section_4_Faust_Law_and_Order_Icon.png</t>
         </is>
       </c>
       <c r="W119" t="n">
@@ -14794,7 +14790,7 @@
       </c>
       <c r="N120" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Zwei%20Assoc.%20South%20Section%204/1120601.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Zwei%20Assoc.%20South%20Section%204/1120601_1.png</t>
         </is>
       </c>
       <c r="O120" t="inlineStr">
@@ -14814,7 +14810,7 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Zwei%20Assoc.%20South%20Section%204/1120601.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Zwei%20Assoc.%20South%20Section%204/1120602_2.png</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
@@ -14834,7 +14830,7 @@
       </c>
       <c r="V120" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Zwei%20Assoc.%20South%20Section%204/1120601.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Zwei%20Assoc.%20South%20Section%204/1120603_3.png</t>
         </is>
       </c>
       <c r="W120" t="n">
@@ -14917,7 +14913,7 @@
       </c>
       <c r="N121" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Molar%20Boatworks%20Fixer/1080701_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Ready_to_Crush_Ishmael_Icon.png/74px-Ready_to_Crush_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="O121" t="inlineStr">
@@ -14937,7 +14933,7 @@
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Molar%20Boatworks%20Fixer/1080701.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Explosive_Blast_Ishmael_Icon.png/74px-Explosive_Blast_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="S121" t="inlineStr">
@@ -14957,7 +14953,7 @@
       </c>
       <c r="V121" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Molar%20Boatworks%20Fixer/1080701.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Risky_Judgement_Ishmael_Icon.png/74px-Risky_Judgement_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="W121" t="n">
@@ -15036,7 +15032,7 @@
       </c>
       <c r="N122" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Molar%20Boatworks%20Fixer/1100701_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Fierce_Assault_Sinclair_Icon.png/74px-Fierce_Assault_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="O122" t="inlineStr">
@@ -15056,7 +15052,7 @@
       </c>
       <c r="R122" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Molar%20Boatworks%20Fixer/1100701.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Steady..._Sinclair_Icon.png/74px-Steady..._Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="S122" t="inlineStr">
@@ -15076,7 +15072,7 @@
       </c>
       <c r="V122" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Molar%20Boatworks%20Fixer/1100701.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Gamble_Sinclair_Icon.png/74px-Gamble_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="W122" t="n">
@@ -15151,7 +15147,7 @@
       </c>
       <c r="N123" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/Cinq%20Assoc.%20South%20Section%205%20Director/1030501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Remise_Don_Quixote_Icon.png/74px-Remise_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="O123" t="inlineStr">
@@ -15171,7 +15167,7 @@
       </c>
       <c r="R123" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/Cinq%20Assoc.%20South%20Section%205%20Director/1030501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Fl%C3%A8che_Don_Quixote_Icon.png/74px-Fl%C3%A8che_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="S123" t="inlineStr">
@@ -15191,7 +15187,7 @@
       </c>
       <c r="V123" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/Cinq%20Assoc.%20South%20Section%205%20Director/1030501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Salut%21_Don_Quixote_Icon.png/74px-Salut%21_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="W123" t="n">
@@ -15274,7 +15270,7 @@
       </c>
       <c r="N124" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/R%20Corp.%204th%20Pack%20Rhino/1050601_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Weighty_Bash_Meursault_Icon.png/74px-Weighty_Bash_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="O124" t="inlineStr">
@@ -15294,7 +15290,7 @@
       </c>
       <c r="R124" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/R%20Corp.%204th%20Pack%20Rhino/1050601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Demolish_Meursault_Icon.png/74px-Demolish_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="S124" t="inlineStr">
@@ -15314,7 +15310,7 @@
       </c>
       <c r="V124" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/R%20Corp.%204th%20Pack%20Rhino/1050601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Rhino_Ram_Meursault_Icon.png/74px-Rhino_Ram_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="W124" t="n">
@@ -15393,7 +15389,7 @@
       </c>
       <c r="N125" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Zwei%20Assoc.%20South%20Section%205/1090601_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Careful_Obstruction_Rodion_Icon.png/74px-Careful_Obstruction_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="O125" t="inlineStr">
@@ -15411,7 +15407,11 @@
           <t>타격</t>
         </is>
       </c>
-      <c r="R125" t="inlineStr"/>
+      <c r="R125" t="inlineStr">
+        <is>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Focused_Defense_Rodion_Icon.png/74px-Focused_Defense_Rodion_Icon.png</t>
+        </is>
+      </c>
       <c r="S125" t="inlineStr">
         <is>
           <t>위협 대상 제압</t>
@@ -15429,7 +15429,7 @@
       </c>
       <c r="V125" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Zwei%20Assoc.%20South%20Section%205/1090601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Subdue_Threat_Rodion_Icon.png/74px-Subdue_Threat_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="W125" t="n">
@@ -15508,7 +15508,7 @@
       </c>
       <c r="N126" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Liu%20Assoc.%20South%20Section%204/1080601_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Red_Kick_Ishmael_Icon.png/74px-Red_Kick_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="O126" t="inlineStr">
@@ -15528,7 +15528,7 @@
       </c>
       <c r="R126" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Liu%20Assoc.%20South%20Section%204/1080601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Frontal_Assault_Ishmael_Icon.png/74px-Frontal_Assault_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="S126" t="inlineStr">
@@ -15548,7 +15548,7 @@
       </c>
       <c r="V126" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Liu%20Assoc.%20South%20Section%204/1080601.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Inner_Gate_Elbow_Strike_Ishmael_Icon.png/74px-Inner_Gate_Elbow_Strike_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="W126" t="n">
@@ -15627,7 +15627,7 @@
       </c>
       <c r="N127" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/K%20Corp.%20Class%203%20Excision%20Staff/1060501_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Impede_the_Intruder_Hong_Lu_Icon.png/74px-Impede_the_Intruder_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="O127" t="inlineStr">
@@ -15647,7 +15647,7 @@
       </c>
       <c r="R127" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/K%20Corp.%20Class%203%20Excision%20Staff/1060501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Decay_Blade_Hong_Lu_Icon.png/74px-Decay_Blade_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="S127" t="inlineStr">
@@ -15667,7 +15667,7 @@
       </c>
       <c r="V127" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/K%20Corp.%20Class%203%20Excision%20Staff/1060501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Excise_Target_Hong_Lu_Icon.png/74px-Excise_Target_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="W127" t="n">
@@ -15766,7 +15766,7 @@
       </c>
       <c r="R128" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Lobotomy%20E.G.O%20Red%20Sheet/1100601.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Lobotomy%20E.G.O%20Red%20Sheet/1100602_2.png</t>
         </is>
       </c>
       <c r="S128" t="inlineStr">
@@ -15786,7 +15786,7 @@
       </c>
       <c r="V128" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Lobotomy%20E.G.O%20Red%20Sheet/1100601.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Lobotomy%20E.G.O%20Red%20Sheet/1100603_3.png</t>
         </is>
       </c>
       <c r="W128" t="n">
@@ -15885,7 +15885,7 @@
       </c>
       <c r="R129" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Effloresced%20E.G.O%20Spicebush/1010401.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Effloresced%20E.G.O%20Spicebush/1010402_2.png</t>
         </is>
       </c>
       <c r="S129" t="inlineStr">
@@ -15905,7 +15905,7 @@
       </c>
       <c r="V129" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Effloresced%20E.G.O%20Spicebush/1010401.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Effloresced%20E.G.O%20Spicebush/1010403_3.png</t>
         </is>
       </c>
       <c r="W129" t="n">
@@ -16008,7 +16008,7 @@
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Lobotomy%20E.G.O%20Sloshing/1080501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Lobotomy%20E.G.O%20Sloshing/1080502_2.png</t>
         </is>
       </c>
       <c r="S130" t="inlineStr">
@@ -16028,7 +16028,7 @@
       </c>
       <c r="V130" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Lobotomy%20E.G.O%20Sloshing/1080501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Lobotomy%20E.G.O%20Sloshing/1080503_3.png</t>
         </is>
       </c>
       <c r="W130" t="n">
@@ -16115,7 +16115,7 @@
       </c>
       <c r="N131" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Lobotomy%20E.G.O%20Sunshower/1070501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Lobotomy%20E.G.O%20Sunshower/1070501_1.png</t>
         </is>
       </c>
       <c r="O131" t="inlineStr">
@@ -16135,7 +16135,7 @@
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Lobotomy%20E.G.O%20Sunshower/1070501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Lobotomy%20E.G.O%20Sunshower/1070502_2.png</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
@@ -16155,7 +16155,7 @@
       </c>
       <c r="V131" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Lobotomy%20E.G.O%20Sunshower/1070501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Lobotomy%20E.G.O%20Sunshower/1070503_3.png</t>
         </is>
       </c>
       <c r="W131" t="n">
@@ -16242,7 +16242,7 @@
       </c>
       <c r="N132" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Rosespanner%20Workshop%20Fixer/1120501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Rosespanner%20Workshop%20Fixer/1120501_1.png</t>
         </is>
       </c>
       <c r="O132" t="inlineStr">
@@ -16262,7 +16262,7 @@
       </c>
       <c r="R132" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Rosespanner%20Workshop%20Fixer/1120501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Rosespanner%20Workshop%20Fixer/1120502_2.png</t>
         </is>
       </c>
       <c r="S132" t="inlineStr">
@@ -16282,7 +16282,7 @@
       </c>
       <c r="V132" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Rosespanner%20Workshop%20Fixer/1120501.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Rosespanner%20Workshop%20Fixer/1120503_3.png</t>
         </is>
       </c>
       <c r="W132" t="n">
@@ -16365,7 +16365,7 @@
       </c>
       <c r="N133" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Rosespanner%20Workshop%20Fixer/1050501_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Saddled_Tasks_Meursault_Icon.png/74px-Saddled_Tasks_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="O133" t="inlineStr">
@@ -16385,7 +16385,7 @@
       </c>
       <c r="R133" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Rosespanner%20Workshop%20Fixer/1050501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Forced_Break_Meursault_Icon.png/74px-Forced_Break_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="S133" t="inlineStr">
@@ -16405,7 +16405,7 @@
       </c>
       <c r="V133" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Rosespanner%20Workshop%20Fixer/1050501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Finishing_Runup_Meursault_Icon.png/74px-Finishing_Runup_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="W133" t="n">
@@ -16488,7 +16488,7 @@
       </c>
       <c r="N134" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Rosespanner%20Workshop%20Rep/1090501_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Rev_Up_Rodion_Icon.png/74px-Rev_Up_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="O134" t="inlineStr">
@@ -16508,7 +16508,7 @@
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Rosespanner%20Workshop%20Rep/1090501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Vibration_Compression_Rodion_Icon.png/74px-Vibration_Compression_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="S134" t="inlineStr">
@@ -16528,7 +16528,7 @@
       </c>
       <c r="V134" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Rosespanner%20Workshop%20Rep/1090501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Let%27s_Rack_Up_Some_Scores_Rodion_Icon.png/74px-Let%27s_Rack_Up_Some_Scores_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="W134" t="n">
@@ -16607,7 +16607,7 @@
       </c>
       <c r="N135" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/N%20Corp.%20Mittelhammer/1030401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Rightful_Purge_Don_Quixote_Icon.png/74px-Rightful_Purge_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="O135" t="inlineStr">
@@ -16627,7 +16627,7 @@
       </c>
       <c r="R135" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/N%20Corp.%20Mittelhammer/1030401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Enactment%21_Don_Quixote_Icon.png/74px-Enactment%21_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="S135" t="inlineStr">
@@ -16647,7 +16647,7 @@
       </c>
       <c r="V135" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/N%20Corp.%20Mittelhammer/1030401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Fanatical_Judgement_Don_Quixote_Icon.png/74px-Fanatical_Judgement_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="W135" t="n">
@@ -16730,7 +16730,7 @@
       </c>
       <c r="N136" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/The%20One%20Who%20Shall%20Grip/1100501_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Coerced_Judgement_Sinclair_Icon.png/74px-Coerced_Judgement_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="O136" t="inlineStr">
@@ -16750,7 +16750,7 @@
       </c>
       <c r="R136" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/The%20One%20Who%20Shall%20Grip/1100501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Amoral_Enactment_Sinclair_Icon.png/74px-Amoral_Enactment_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="S136" t="inlineStr">
@@ -16770,7 +16770,7 @@
       </c>
       <c r="V136" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/The%20One%20Who%20Shall%20Grip/1100501.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Self-destructive_Purge_Sinclair_Icon.png/74px-Self-destructive_Purge_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="W136" t="n">
@@ -16849,7 +16849,7 @@
       </c>
       <c r="N137" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/R.B.%20Chef%20de%20Cuisine/1040401_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/P.C._Ry%C5%8Dsh%C5%AB_Icon.png/74px-P.C._Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="O137" t="inlineStr">
@@ -16869,7 +16869,7 @@
       </c>
       <c r="R137" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/R.B.%20Chef%20de%20Cuisine/1040401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/I.H._Ry%C5%8Dsh%C5%AB_Icon.png/74px-I.H._Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="S137" t="inlineStr">
@@ -16889,7 +16889,7 @@
       </c>
       <c r="V137" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/R.B.%20Chef%20de%20Cuisine/1040401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/I_Can_Cook_Anything_Ry%C5%8Dsh%C5%AB_Icon.png/74px-I_Can_Cook_Anything_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="W137" t="n">
@@ -16968,7 +16968,7 @@
       </c>
       <c r="N138" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/R.B.%20Sous-chef/1120401.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/R.B.%20Sous-chef/1120401_1.png</t>
         </is>
       </c>
       <c r="O138" t="inlineStr">
@@ -16988,7 +16988,7 @@
       </c>
       <c r="R138" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/R.B.%20Sous-chef/1120401.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/R.B.%20Sous-chef/1120402_2.png</t>
         </is>
       </c>
       <c r="S138" t="inlineStr">
@@ -17008,7 +17008,7 @@
       </c>
       <c r="V138" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/R.B.%20Sous-chef/1120401.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/R.B.%20Sous-chef/1120403_3.png</t>
         </is>
       </c>
       <c r="W138" t="n">
@@ -17087,7 +17087,7 @@
       </c>
       <c r="N139" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Liu%20Assoc.%20South%20Section%205/1060401_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Warm_Up_Hong_Lu_Icon.png/74px-Warm_Up_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="O139" t="inlineStr">
@@ -17107,7 +17107,7 @@
       </c>
       <c r="R139" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Liu%20Assoc.%20South%20Section%205/1060401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Flowing_Flame_Hong_Lu_Icon.png/74px-Flowing_Flame_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="S139" t="inlineStr">
@@ -17127,7 +17127,7 @@
       </c>
       <c r="V139" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Liu%20Assoc.%20South%20Section%205/1060401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Crimson_Blaze_Fist_Hong_Lu_Icon.png/74px-Crimson_Blaze_Fist_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="W139" t="n">
@@ -17206,7 +17206,7 @@
       </c>
       <c r="N140" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/Seven%20Assoc.%20South%20Section%206%20Director/1110401_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Predictive_Analysis_Outis_Icon.png/74px-Predictive_Analysis_Outis_Icon.png</t>
         </is>
       </c>
       <c r="O140" t="inlineStr">
@@ -17226,7 +17226,7 @@
       </c>
       <c r="R140" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/Seven%20Assoc.%20South%20Section%206%20Director/1110401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Field_Command_Outis_Icon.png/74px-Field_Command_Outis_Icon.png</t>
         </is>
       </c>
       <c r="S140" t="inlineStr">
@@ -17246,7 +17246,7 @@
       </c>
       <c r="V140" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/Seven%20Assoc.%20South%20Section%206%20Director/1110401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Exploit_the_Gap_Outis_Icon.png/74px-Exploit_the_Gap_Outis_Icon.png</t>
         </is>
       </c>
       <c r="W140" t="n">
@@ -17325,7 +17325,7 @@
       </c>
       <c r="N141" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/The%20One%20Who%20Grips/1020401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Cackle_Faust_Icon.png/74px-Cackle_Faust_Icon.png</t>
         </is>
       </c>
       <c r="O141" t="inlineStr">
@@ -17345,7 +17345,7 @@
       </c>
       <c r="R141" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/The%20One%20Who%20Grips/1020401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/The_Gripping_Faust_Icon.png/74px-The_Gripping_Faust_Icon.png</t>
         </is>
       </c>
       <c r="S141" t="inlineStr">
@@ -17365,7 +17365,7 @@
       </c>
       <c r="V141" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/The%20One%20Who%20Grips/1020401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Execution_Faust_Icon.png/74px-Execution_Faust_Icon.png</t>
         </is>
       </c>
       <c r="W141" t="n">
@@ -17444,7 +17444,7 @@
       </c>
       <c r="N142" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/N%20Corp.%20Kleinhammer/1070401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Gawky_Nailing_Heathcliff_Icon.png/74px-Gawky_Nailing_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="O142" t="inlineStr">
@@ -17464,7 +17464,7 @@
       </c>
       <c r="R142" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/N%20Corp.%20Kleinhammer/1070401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Puri...fy%21_Heathcliff_Icon.png/74px-Puri...fy%21_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="S142" t="inlineStr">
@@ -17484,7 +17484,7 @@
       </c>
       <c r="V142" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/N%20Corp.%20Kleinhammer/1070401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Infirm_Retribution_Heathcliff_Icon.png/74px-Infirm_Retribution_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="W142" t="n">
@@ -17559,7 +17559,7 @@
       </c>
       <c r="N143" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/N%20Corp.%20Gro%C3%9Fhammer/1050401_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Drive_Meursault_Icon.png/74px-Drive_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="O143" t="inlineStr">
@@ -17579,7 +17579,7 @@
       </c>
       <c r="R143" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/N%20Corp.%20Gro%C3%9Fhammer/1050401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/You_Are_Cleansed_of_Sin_Meursault_Icon.png/74px-You_Are_Cleansed_of_Sin_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="S143" t="inlineStr">
@@ -17599,7 +17599,7 @@
       </c>
       <c r="V143" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/N%20Corp.%20Gro%C3%9Fhammer/1050401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Annihilate_Heretics_Meursault_Icon.png/74px-Annihilate_Heretics_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="W143" t="n">
@@ -17678,7 +17678,7 @@
       </c>
       <c r="N144" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/N%20Corp.%20Mittelhammer/1090401_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Devoted_Hammering_Rodion_Icon.png/74px-Devoted_Hammering_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="O144" t="inlineStr">
@@ -17698,7 +17698,7 @@
       </c>
       <c r="R144" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/N%20Corp.%20Mittelhammer/1090401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Zealous_Purge_Rodion_Icon.png/74px-Zealous_Purge_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="S144" t="inlineStr">
@@ -17718,7 +17718,7 @@
       </c>
       <c r="V144" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/N%20Corp.%20Mittelhammer/1090401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Ironclad_Retribution_Rodion_Icon.png/74px-Ironclad_Retribution_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="W144" t="n">
@@ -17797,7 +17797,7 @@
       </c>
       <c r="N145" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Blade%20Lineage%20Salsu/1010301_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Striker%27s_Stance_Yi_Sang_Icon.png/74px-Striker%27s_Stance_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="O145" t="inlineStr">
@@ -17817,7 +17817,7 @@
       </c>
       <c r="R145" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Blade%20Lineage%20Salsu/1010301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Heel_Turn_Yi_Sang_Icon.png/74px-Heel_Turn_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="S145" t="inlineStr">
@@ -17837,7 +17837,7 @@
       </c>
       <c r="V145" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Blade%20Lineage%20Salsu/1010301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Flank_Thrust_Yi_Sang_Icon.png/74px-Flank_Thrust_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="W145" t="n">
@@ -17916,7 +17916,7 @@
       </c>
       <c r="N146" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Seven%20Assoc.%20South%20Section%206/1010201_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Fl%C3%A8che_Yi_Sang_Icon.png/74px-Fl%C3%A8che_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="O146" t="inlineStr">
@@ -17936,7 +17936,7 @@
       </c>
       <c r="R146" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Seven%20Assoc.%20South%20Section%206/1010201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Riposte_Yi_Sang_Icon.png/74px-Riposte_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="S146" t="inlineStr">
@@ -17956,7 +17956,7 @@
       </c>
       <c r="V146" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/Seven%20Assoc.%20South%20Section%206/1010201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Moulinet_Yi_Sang_Icon.png/74px-Moulinet_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="W146" t="n">
@@ -18035,7 +18035,7 @@
       </c>
       <c r="N147" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/LCB%20Sinner/1010101_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Deflect_Yi_Sang_Icon.png/74px-Deflect_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="O147" t="inlineStr">
@@ -18055,7 +18055,7 @@
       </c>
       <c r="R147" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/LCB%20Sinner/1010101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/End-stop_Stab_Yi_Sang_Icon.png/74px-End-stop_Stab_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="S147" t="inlineStr">
@@ -18075,7 +18075,7 @@
       </c>
       <c r="V147" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Yi%20Sang/LCB%20Sinner/1010101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Enjamb_Yi_Sang_Icon.png/74px-Enjamb_Yi_Sang_Icon.png</t>
         </is>
       </c>
       <c r="W147" t="n">
@@ -18148,7 +18148,11 @@
           <t>타격</t>
         </is>
       </c>
-      <c r="N148" t="inlineStr"/>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Energy_Cycle_Faust_Icon.png/74px-Energy_Cycle_Faust_Icon.png</t>
+        </is>
+      </c>
       <c r="O148" t="inlineStr">
         <is>
           <t>도약</t>
@@ -18164,7 +18168,11 @@
           <t>타격</t>
         </is>
       </c>
-      <c r="R148" t="inlineStr"/>
+      <c r="R148" t="inlineStr">
+        <is>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Leap_Faust_Icon.png/74px-Leap_Faust_Icon.png</t>
+        </is>
+      </c>
       <c r="S148" t="inlineStr">
         <is>
           <t>과충전</t>
@@ -18180,7 +18188,11 @@
           <t>타격</t>
         </is>
       </c>
-      <c r="V148" t="inlineStr"/>
+      <c r="V148" t="inlineStr">
+        <is>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Overcharge_Faust_Icon.png/74px-Overcharge_Faust_Icon.png</t>
+        </is>
+      </c>
       <c r="W148" t="n">
         <v>2</v>
       </c>
@@ -18259,7 +18271,11 @@
           <t>참격</t>
         </is>
       </c>
-      <c r="N149" t="inlineStr"/>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Sole_Strike_Faust_Icon.png/74px-Sole_Strike_Faust_Icon.png</t>
+        </is>
+      </c>
       <c r="O149" t="inlineStr">
         <is>
           <t>깊게베기</t>
@@ -18275,7 +18291,11 @@
           <t>참격</t>
         </is>
       </c>
-      <c r="R149" t="inlineStr"/>
+      <c r="R149" t="inlineStr">
+        <is>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Deep_Cuts_Faust_Icon.png/74px-Deep_Cuts_Faust_Icon.png</t>
+        </is>
+      </c>
       <c r="S149" t="inlineStr">
         <is>
           <t>기회 노리기</t>
@@ -18291,7 +18311,11 @@
           <t>참격</t>
         </is>
       </c>
-      <c r="V149" t="inlineStr"/>
+      <c r="V149" t="inlineStr">
+        <is>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Opportunistic_Slash_Faust_Icon.png/74px-Opportunistic_Slash_Faust_Icon.png</t>
+        </is>
+      </c>
       <c r="W149" t="n">
         <v>3</v>
       </c>
@@ -18364,7 +18388,7 @@
       </c>
       <c r="N150" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/LCB%20Sinner/1020101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Downward_Slash_Faust_Icon.png/74px-Downward_Slash_Faust_Icon.png</t>
         </is>
       </c>
       <c r="O150" t="inlineStr">
@@ -18384,7 +18408,7 @@
       </c>
       <c r="R150" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/LCB%20Sinner/1020101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Upward_Slash_Faust_Icon.png/74px-Upward_Slash_Faust_Icon.png</t>
         </is>
       </c>
       <c r="S150" t="inlineStr">
@@ -18404,7 +18428,7 @@
       </c>
       <c r="V150" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Faust/LCB%20Sinner/1020101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Drilling_Stab_Faust_Icon.png/74px-Drilling_Stab_Faust_Icon.png</t>
         </is>
       </c>
       <c r="W150" t="n">
@@ -18483,7 +18507,7 @@
       </c>
       <c r="N151" t="inlineStr">
         <is>
-          <t>https://cdn.discordapp.com/avatars/710417870152269834/c846322deab86bee0b1b25b4dc00ec7a.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Rip_Don_Quixote_Icon.png/74px-Rip_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="O151" t="inlineStr">
@@ -18503,7 +18527,7 @@
       </c>
       <c r="R151" t="inlineStr">
         <is>
-          <t>https://cdn.discordapp.com/avatars/710417870152269834/c846322deab86bee0b1b25b4dc00ec7a.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Leap_Don_Quixote_Icon.png/74px-Leap_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="S151" t="inlineStr">
@@ -18523,7 +18547,7 @@
       </c>
       <c r="V151" t="inlineStr">
         <is>
-          <t>https://cdn.discordapp.com/avatars/710417870152269834/c846322deab86bee0b1b25b4dc00ec7a.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Rip_Space_Don_Quixote_Icon.png/74px-Rip_Space_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="W151" t="n">
@@ -18602,7 +18626,7 @@
       </c>
       <c r="N152" t="inlineStr">
         <is>
-          <t>https://cdn.discordapp.com/avatars/1306147695815163905/2a5c1a9d0a1b797becaab23de19ca19d.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Catch_Breath_Don_Quixote_Icon.png/74px-Catch_Breath_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="O152" t="inlineStr">
@@ -18622,7 +18646,7 @@
       </c>
       <c r="R152" t="inlineStr">
         <is>
-          <t>https://cdn.discordapp.com/avatars/1306147695815163905/2a5c1a9d0a1b797becaab23de19ca19d.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Dual_Strike_Don_Quixote_Icon.png/74px-Dual_Strike_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="S152" t="inlineStr">
@@ -18642,7 +18666,7 @@
       </c>
       <c r="V152" t="inlineStr">
         <is>
-          <t>https://cdn.discordapp.com/avatars/1306147695815163905/2a5c1a9d0a1b797becaab23de19ca19d.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Overbreathe_Don_Quixote_Icon.png/74px-Overbreathe_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="W152" t="n">
@@ -18721,7 +18745,7 @@
       </c>
       <c r="N153" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/LCB%20Sinner/1030101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Joust_Don_Quixote_Icon.png/74px-Joust_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="O153" t="inlineStr">
@@ -18741,7 +18765,7 @@
       </c>
       <c r="R153" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/LCB%20Sinner/1030101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Galloping_Tilt_Don_Quixote_Icon.png/74px-Galloping_Tilt_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="S153" t="inlineStr">
@@ -18761,7 +18785,7 @@
       </c>
       <c r="V153" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Don%20Quixote/LCB%20Sinner/1030101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/For_Justice%21_Don_Quixote_Icon.png/74px-For_Justice%21_Don_Quixote_Icon.png</t>
         </is>
       </c>
       <c r="W153" t="n">
@@ -18836,7 +18860,7 @@
       </c>
       <c r="N154" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Kurokumo%20Clan%20Wakashu/1040301_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Focus_Strike_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Focus_Strike_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="O154" t="inlineStr">
@@ -18856,7 +18880,7 @@
       </c>
       <c r="R154" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Kurokumo%20Clan%20Wakashu/1040301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Clean_Up_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Clean_Up_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="S154" t="inlineStr">
@@ -18876,7 +18900,7 @@
       </c>
       <c r="V154" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Kurokumo%20Clan%20Wakashu/1040301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Lenticular_Swirl_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Lenticular_Swirl_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="W154" t="n">
@@ -18955,7 +18979,7 @@
       </c>
       <c r="N155" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/Seven_Assoc._South_Section_6/1040201_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Slash_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Slash_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="O155" t="inlineStr">
@@ -18973,7 +18997,11 @@
           <t>타격</t>
         </is>
       </c>
-      <c r="R155" t="inlineStr"/>
+      <c r="R155" t="inlineStr">
+        <is>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Upper_Slash_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Upper_Slash_Ry%C5%8Dsh%C5%AB_Icon.png</t>
+        </is>
+      </c>
       <c r="S155" t="inlineStr">
         <is>
           <t>스워시</t>
@@ -18989,7 +19017,11 @@
           <t>타격</t>
         </is>
       </c>
-      <c r="V155" t="inlineStr"/>
+      <c r="V155" t="inlineStr">
+        <is>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Swash_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Swash_Ry%C5%8Dsh%C5%AB_Icon.png</t>
+        </is>
+      </c>
       <c r="W155" t="n">
         <v>3</v>
       </c>
@@ -19066,7 +19098,7 @@
       </c>
       <c r="N156" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/LCB%20Sinner/1040101_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Paint_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Paint_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="O156" t="inlineStr">
@@ -19086,7 +19118,7 @@
       </c>
       <c r="R156" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/LCB%20Sinner/1040101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Splatter_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Splatter_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="S156" t="inlineStr">
@@ -19106,7 +19138,7 @@
       </c>
       <c r="V156" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ryoshu/LCB%20Sinner/1040101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Brushstroke_Ry%C5%8Dsh%C5%AB_Icon.png/74px-Brushstroke_Ry%C5%8Dsh%C5%AB_Icon.png</t>
         </is>
       </c>
       <c r="W156" t="n">
@@ -19185,7 +19217,7 @@
       </c>
       <c r="N157" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/W%20Corp.%20Cleanup%20Crew/1050301_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Rip_Meursault_Icon.png/74px-Rip_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="O157" t="inlineStr">
@@ -19205,7 +19237,7 @@
       </c>
       <c r="R157" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/W%20Corp.%20Cleanup%20Crew/1050301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Energy_Cycle_Meursault_Icon.png/74px-Energy_Cycle_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="S157" t="inlineStr">
@@ -19225,7 +19257,7 @@
       </c>
       <c r="V157" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/W%20Corp.%20Cleanup%20Crew/1050301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Energy_Current_Meursault_Icon.png/74px-Energy_Current_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="W157" t="n">
@@ -19304,7 +19336,7 @@
       </c>
       <c r="N158" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Liu%20Assoc.%20South%20Section%206/1050201_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Assault_Meursault_Icon.png/74px-Assault_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="O158" t="inlineStr">
@@ -19324,7 +19356,7 @@
       </c>
       <c r="R158" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Liu%20Assoc.%20South%20Section%206/1050201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Stalwart_Stance_Meursault_Icon.png/74px-Stalwart_Stance_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="S158" t="inlineStr">
@@ -19344,7 +19376,7 @@
       </c>
       <c r="V158" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/Liu%20Assoc.%20South%20Section%206/1050201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Perfected_Death_Fist_Meursault_Icon.png/74px-Perfected_Death_Fist_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="W158" t="n">
@@ -19423,7 +19455,7 @@
       </c>
       <c r="N159" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/LCB%20Sinner/1050101_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Un%2C_Deux_Meursault_Icon.png/74px-Un%2C_Deux_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="O159" t="inlineStr">
@@ -19443,7 +19475,7 @@
       </c>
       <c r="R159" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/LCB%20Sinner/1050101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Nailing_Fist_Meursault_Icon.png/74px-Nailing_Fist_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="S159" t="inlineStr">
@@ -19463,7 +19495,7 @@
       </c>
       <c r="V159" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Meursault/LCB%20Sinner/1050101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Des_Coups_Meursault_Icon.png/74px-Des_Coups_Meursault_Icon.png</t>
         </is>
       </c>
       <c r="W159" t="n">
@@ -19538,7 +19570,7 @@
       </c>
       <c r="N160" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Tingtang%20Gang%20Gangleader/1060301_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Throat_Slit_Hong_Lu_Icon.png/74px-Throat_Slit_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="O160" t="inlineStr">
@@ -19558,7 +19590,7 @@
       </c>
       <c r="R160" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Tingtang%20Gang%20Gangleader/1060301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Shank_Hong_Lu_Icon.png/74px-Shank_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="S160" t="inlineStr">
@@ -19578,7 +19610,7 @@
       </c>
       <c r="V160" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Tingtang%20Gang%20Gangleader/1060301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Mutilate_Hong_Lu_Icon.png/74px-Mutilate_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="W160" t="n">
@@ -19657,7 +19689,7 @@
       </c>
       <c r="N161" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Kurokumo%20Clan%20Wakashu/1060201_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Cleave_Hong_Lu_Icon.png/74px-Cleave_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="O161" t="inlineStr">
@@ -19677,7 +19709,7 @@
       </c>
       <c r="R161" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Kurokumo%20Clan%20Wakashu/1060201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Cloud_Cutter_Hong_Lu_Icon.png/74px-Cloud_Cutter_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="S161" t="inlineStr">
@@ -19697,7 +19729,7 @@
       </c>
       <c r="V161" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/Kurokumo%20Clan%20Wakashu/1060201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Cloudburst_Hong_Lu_Icon.png/74px-Cloudburst_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="W161" t="n">
@@ -19780,7 +19812,7 @@
       </c>
       <c r="N162" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/LCB%20Sinner/1060101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Downward_Cleave_Hong_Lu_Icon.png/74px-Downward_Cleave_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="O162" t="inlineStr">
@@ -19800,7 +19832,7 @@
       </c>
       <c r="R162" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/LCB%20Sinner/1060101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Dual_Strike_Hong_Lu_Icon.png/74px-Dual_Strike_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="S162" t="inlineStr">
@@ -19820,7 +19852,7 @@
       </c>
       <c r="V162" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Hong%20Lu/LCB%20Sinner/1060101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Whirlwind_Hong_Lu_Icon.png/74px-Whirlwind_Hong_Lu_Icon.png</t>
         </is>
       </c>
       <c r="W162" t="n">
@@ -19903,7 +19935,7 @@
       </c>
       <c r="N163" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/R%20Corp.%204th%20Pack%20Rabbit/1070301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Graze_the_Grass_Heathcliff_Icon.png/74px-Graze_the_Grass_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="O163" t="inlineStr">
@@ -19923,7 +19955,7 @@
       </c>
       <c r="R163" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/R%20Corp.%204th%20Pack%20Rabbit/1070301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Concentrated_Fire_Heathcliff_Icon.png/74px-Concentrated_Fire_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="S163" t="inlineStr">
@@ -19943,7 +19975,7 @@
       </c>
       <c r="V163" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/R%20Corp.%204th%20Pack%20Rabbit/1070301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Quick_Suppression_Heathcliff_Icon.png/74px-Quick_Suppression_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="W163" t="n">
@@ -20022,7 +20054,7 @@
       </c>
       <c r="N164" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Shi%20Assoc.%20South%20Section%205/1070201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Extreme_Edge_Heathcliff_Icon.png/74px-Extreme_Edge_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="O164" t="inlineStr">
@@ -20042,7 +20074,7 @@
       </c>
       <c r="R164" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Shi%20Assoc.%20South%20Section%205/1070201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Flying_Sword_Heathcliff_Icon.png/74px-Flying_Sword_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="S164" t="inlineStr">
@@ -20062,7 +20094,7 @@
       </c>
       <c r="V164" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/Shi%20Assoc.%20South%20Section%205/1070201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Flashing_Strike_Heathcliff_Icon.png/74px-Flashing_Strike_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="W164" t="n">
@@ -20141,7 +20173,7 @@
       </c>
       <c r="N165" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/LCB%20Sinner/1070101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Bat_Bash_Heathcliff_Icon.png/74px-Bat_Bash_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="O165" t="inlineStr">
@@ -20161,7 +20193,7 @@
       </c>
       <c r="R165" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/LCB%20Sinner/1070101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Smackdown_Heathcliff_Icon.png/74px-Smackdown_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="S165" t="inlineStr">
@@ -20181,7 +20213,7 @@
       </c>
       <c r="V165" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Heathcliff/LCB%20Sinner/1070101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Upheaval_Heathcliff_Icon.png/74px-Upheaval_Heathcliff_Icon.png</t>
         </is>
       </c>
       <c r="W165" t="n">
@@ -20260,7 +20292,7 @@
       </c>
       <c r="N166" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/R%20Corp.%204th%20Pack%20Reindeer/1080201_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Mind_Strike_Ishmael_Icon.png/74px-Mind_Strike_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="O166" t="inlineStr">
@@ -20280,7 +20312,7 @@
       </c>
       <c r="R166" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/R%20Corp.%204th%20Pack%20Reindeer/1080201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Flaying_Surge_Ishmael_Icon.png/74px-Flaying_Surge_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="S166" t="inlineStr">
@@ -20300,7 +20332,7 @@
       </c>
       <c r="V166" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/R%20Corp.%204th%20Pack%20Reindeer/1080201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Mind_Whip_Ishmael_Icon.png/74px-Mind_Whip_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="W166" t="n">
@@ -20379,7 +20411,7 @@
       </c>
       <c r="N167" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Shi%20Assoc.%20South%20Section%205/1080301_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Flying_Sword_Ishmael_Icon.png/74px-Flying_Sword_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="O167" t="inlineStr">
@@ -20399,7 +20431,7 @@
       </c>
       <c r="R167" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Shi%20Assoc.%20South%20Section%205/1080301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Flashing_Strike_Ishmael_Icon.png/74px-Flashing_Strike_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="S167" t="inlineStr">
@@ -20419,7 +20451,7 @@
       </c>
       <c r="V167" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/Shi%20Assoc.%20South%20Section%205/1080301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Catch_Breath_Ishmael_Icon.png/74px-Catch_Breath_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="W167" t="n">
@@ -20502,7 +20534,7 @@
       </c>
       <c r="N168" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/LCCB%20Assistant%20Manager/1080401_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Shove_Ishmael_Icon.png/74px-Shove_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="O168" t="inlineStr">
@@ -20522,7 +20554,7 @@
       </c>
       <c r="R168" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/LCCB%20Assistant%20Manager/1080401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Quake_Rounds_Ishmael_Icon.png/74px-Quake_Rounds_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="S168" t="inlineStr">
@@ -20542,7 +20574,7 @@
       </c>
       <c r="V168" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/LCCB%20Assistant%20Manager/1080401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Suppress_Ishmael_Icon.png/74px-Suppress_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="W168" t="n">
@@ -20621,7 +20653,7 @@
       </c>
       <c r="N169" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/LCB%20Sinner/1080101_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Loggerhead_Ishmael_Icon.png/74px-Loggerhead_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="O169" t="inlineStr">
@@ -20641,7 +20673,7 @@
       </c>
       <c r="R169" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/LCB%20Sinner/1080101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Slide_Ishmael_Icon.png/74px-Slide_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="S169" t="inlineStr">
@@ -20661,7 +20693,7 @@
       </c>
       <c r="V169" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Ishmael/LCB%20Sinner/1080101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Shield_Bash_Ishmael_Icon.png/74px-Shield_Bash_Ishmael_Icon.png</t>
         </is>
       </c>
       <c r="W169" t="n">
@@ -20750,7 +20782,11 @@
           <t>참격</t>
         </is>
       </c>
-      <c r="R170" t="inlineStr"/>
+      <c r="R170" t="inlineStr">
+        <is>
+          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Kurokumo%20Henchwoman/1090202_2.png</t>
+        </is>
+      </c>
       <c r="S170" t="inlineStr">
         <is>
           <t>쾌청 베기</t>
@@ -20762,7 +20798,11 @@
           <t>참격</t>
         </is>
       </c>
-      <c r="V170" t="inlineStr"/>
+      <c r="V170" t="inlineStr">
+        <is>
+          <t>https://baslimbus.info/assets/drive/sinners/Rodion/Kurokumo%20Henchwoman/1090203_3.png</t>
+        </is>
+      </c>
       <c r="W170" t="n">
         <v>2</v>
       </c>
@@ -20835,7 +20875,7 @@
       </c>
       <c r="N171" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/LCCB%20Assistant%20Manager/1090301_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Bludgeon_Rodion_Icon.png/74px-Bludgeon_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="O171" t="inlineStr">
@@ -20855,7 +20895,7 @@
       </c>
       <c r="R171" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/LCCB%20Assistant%20Manager/1090301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Thrust_Rodion_Icon.png/74px-Thrust_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="S171" t="inlineStr">
@@ -20875,7 +20915,7 @@
       </c>
       <c r="V171" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/LCCB%20Assistant%20Manager/1090301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Suppress_Rodion_Icon.png/74px-Suppress_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="W171" t="n">
@@ -20954,7 +20994,7 @@
       </c>
       <c r="N172" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/LCB%20Sinner/1090101_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Strike_Down_Rodion_Icon.png/74px-Strike_Down_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="O172" t="inlineStr">
@@ -20974,7 +21014,7 @@
       </c>
       <c r="R172" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/LCB%20Sinner/1090101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Axe_Combo_Rodion_Icon.png/74px-Axe_Combo_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="S172" t="inlineStr">
@@ -20994,7 +21034,7 @@
       </c>
       <c r="V172" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Rodion/LCB%20Sinner/1090101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Slay_Rodion_Icon.png/74px-Slay_Rodion_Icon.png</t>
         </is>
       </c>
       <c r="W172" t="n">
@@ -21073,7 +21113,7 @@
       </c>
       <c r="N173" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Blade%20Lineage%20Salsu/1100201_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Slice_then_Stab_Sinclair_Icon.png/74px-Slice_then_Stab_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="O173" t="inlineStr">
@@ -21093,7 +21133,7 @@
       </c>
       <c r="R173" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Blade%20Lineage%20Salsu/1100201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Slash_Series_Sinclair_Icon.png/74px-Slash_Series_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="S173" t="inlineStr">
@@ -21113,7 +21153,7 @@
       </c>
       <c r="V173" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Blade%20Lineage%20Salsu/1100201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/To_Claim_Their_Bones_Sinclair_Icon.png/74px-To_Claim_Their_Bones_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="W173" t="n">
@@ -21192,7 +21232,7 @@
       </c>
       <c r="N174" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Zwei%20Assoc.%20South%20Section%206/1100301_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Baton_Sinclair_Icon.png/74px-Baton_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="O174" t="inlineStr">
@@ -21212,7 +21252,7 @@
       </c>
       <c r="R174" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Zwei%20Assoc.%20South%20Section%206/1100301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Suppress_Sinclair_Icon.png/74px-Suppress_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="S174" t="inlineStr">
@@ -21232,7 +21272,7 @@
       </c>
       <c r="V174" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Zwei%20Assoc.%20South%20Section%206/1100301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Strong_Strike_Sinclair_Icon.png/74px-Strong_Strike_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="W174" t="n">
@@ -21315,7 +21355,7 @@
       </c>
       <c r="N175" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Los%20Mariachis%20Jefe/1100401_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Baile_y_Rola_Sinclair_Icon.png/74px-Baile_y_Rola_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="O175" t="inlineStr">
@@ -21335,7 +21375,7 @@
       </c>
       <c r="R175" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Los%20Mariachis%20Jefe/1100401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Danza_de_Pasion_Sinclair_Icon.png/74px-Danza_de_Pasion_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="S175" t="inlineStr">
@@ -21355,7 +21395,7 @@
       </c>
       <c r="V175" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/Los%20Mariachis%20Jefe/1100401.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Panata_Party_Sinclair_Icon.png/74px-Panata_Party_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="W175" t="n">
@@ -21434,7 +21474,7 @@
       </c>
       <c r="N176" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/LCB%20Sinner/1100101_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Downward_Swing_Sinclair_Icon.png/74px-Downward_Swing_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="O176" t="inlineStr">
@@ -21454,7 +21494,7 @@
       </c>
       <c r="R176" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/LCB%20Sinner/1100101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Halberd_Combo_Sinclair_Icon.png/74px-Halberd_Combo_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="S176" t="inlineStr">
@@ -21474,7 +21514,7 @@
       </c>
       <c r="V176" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Sinclair/LCB%20Sinner/1100101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Ravaging_Cut_Sinclair_Icon.png/74px-Ravaging_Cut_Sinclair_Icon.png</t>
         </is>
       </c>
       <c r="W176" t="n">
@@ -21549,7 +21589,7 @@
       </c>
       <c r="N177" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/Blade%20Lineage%20Salsu/1110201_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Draw_of_the_Sword_Outis_Icon.png/74px-Draw_of_the_Sword_Outis_Icon.png</t>
         </is>
       </c>
       <c r="O177" t="inlineStr">
@@ -21569,7 +21609,7 @@
       </c>
       <c r="R177" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/Blade%20Lineage%20Salsu/1110201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Acupuncture_Outis_Icon.png/74px-Acupuncture_Outis_Icon.png</t>
         </is>
       </c>
       <c r="S177" t="inlineStr">
@@ -21589,7 +21629,7 @@
       </c>
       <c r="V177" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/Blade%20Lineage%20Salsu/1110201.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Decisive_Dive_Outis_Icon.png/74px-Decisive_Dive_Outis_Icon.png</t>
         </is>
       </c>
       <c r="W177" t="n">
@@ -21668,7 +21708,7 @@
       </c>
       <c r="N178" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/G%20Corp.%20Head%20Manager/1110301_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Order_Outis_Icon.png/74px-Order_Outis_Icon.png</t>
         </is>
       </c>
       <c r="O178" t="inlineStr">
@@ -21688,7 +21728,7 @@
       </c>
       <c r="R178" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/G%20Corp.%20Head%20Manager/1110301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Onslaught_Command_Outis_Icon.png/74px-Onslaught_Command_Outis_Icon.png</t>
         </is>
       </c>
       <c r="S178" t="inlineStr">
@@ -21708,7 +21748,7 @@
       </c>
       <c r="V178" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/G%20Corp.%20Head%20Manager/1110301.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Focus_Outis_Icon.png/74px-Focus_Outis_Icon.png</t>
         </is>
       </c>
       <c r="W178" t="n">
@@ -21787,7 +21827,7 @@
       </c>
       <c r="N179" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/LCB%20Sinner/1110101_1.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Pulled_Blade_Outis_Icon.png/74px-Pulled_Blade_Outis_Icon.png</t>
         </is>
       </c>
       <c r="O179" t="inlineStr">
@@ -21807,7 +21847,7 @@
       </c>
       <c r="R179" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/LCB%20Sinner/1110101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Backslash_Outis_Icon.png/74px-Backslash_Outis_Icon.png</t>
         </is>
       </c>
       <c r="S179" t="inlineStr">
@@ -21827,7 +21867,7 @@
       </c>
       <c r="V179" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Outis/LCB%20Sinner/1110101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Piercing_Thrust_Outis_Icon.png/74px-Piercing_Thrust_Outis_Icon.png</t>
         </is>
       </c>
       <c r="W179" t="n">
@@ -21902,7 +21942,7 @@
       </c>
       <c r="N180" t="inlineStr">
         <is>
-          <t>https://cdn.discordapp.com/avatars/444470393605062656/6fd07f464cbf7f553c7425ac80caa2c8.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/G%20Corp.%20Corporal%20Manager/1120301_1.png</t>
         </is>
       </c>
       <c r="O180" t="inlineStr">
@@ -21922,7 +21962,7 @@
       </c>
       <c r="R180" t="inlineStr">
         <is>
-          <t>https://cdn.discordapp.com/avatars/444470393605062656/6fd07f464cbf7f553c7425ac80caa2c8.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/G%20Corp.%20Corporal%20Manager/1120302_2.png</t>
         </is>
       </c>
       <c r="S180" t="inlineStr">
@@ -21942,7 +21982,7 @@
       </c>
       <c r="V180" t="inlineStr">
         <is>
-          <t>https://cdn.discordapp.com/avatars/444470393605062656/6fd07f464cbf7f553c7425ac80caa2c8.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/G%20Corp.%20Corporal%20Manager/1120303_3.png</t>
         </is>
       </c>
       <c r="W180" t="n">
@@ -22021,7 +22061,7 @@
       </c>
       <c r="N181" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Liu%20Assoc.%20South%20Section%206/1120201.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Liu%20Assoc.%20South%20Section%206/1120201_1.png</t>
         </is>
       </c>
       <c r="O181" t="inlineStr">
@@ -22041,7 +22081,7 @@
       </c>
       <c r="R181" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Liu%20Assoc.%20South%20Section%206/1120201.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Liu%20Assoc.%20South%20Section%206/1120202_2.png</t>
         </is>
       </c>
       <c r="S181" t="inlineStr">
@@ -22061,7 +22101,7 @@
       </c>
       <c r="V181" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Liu%20Assoc.%20South%20Section%206/1120201.png</t>
+          <t>https://baslimbus.info/assets/drive/sinners/Gregor/Liu%20Assoc.%20South%20Section%206/1120203_3.png</t>
         </is>
       </c>
       <c r="W181" t="n">
@@ -22140,7 +22180,7 @@
       </c>
       <c r="N182" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/LCB%20Sinner/1120101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Swipe_Gregor_Icon.png/74px-Swipe_Gregor_Icon.png</t>
         </is>
       </c>
       <c r="O182" t="inlineStr">
@@ -22160,7 +22200,7 @@
       </c>
       <c r="R182" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/LCB%20Sinner/1120101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Jag_Gregor_Icon.png/74px-Jag_Gregor_Icon.png</t>
         </is>
       </c>
       <c r="S182" t="inlineStr">
@@ -22180,7 +22220,7 @@
       </c>
       <c r="V182" t="inlineStr">
         <is>
-          <t>https://baslimbus.info/assets/drive/sinners/Gregor/LCB%20Sinner/1120101.png</t>
+          <t>https://limbuscompany.wiki.gg/images/thumb/Chop_Up_Gregor_Icon.png/74px-Chop_Up_Gregor_Icon.png</t>
         </is>
       </c>
       <c r="W182" t="n">

</xml_diff>